<commit_message>
Corrige instalacao automatica de plotly/openpyxl no Streamlit Cloud e adiciona experimento RAG Fichamento JEV
</commit_message>
<xml_diff>
--- a/Experimento/Conjunto de Testes.xlsx
+++ b/Experimento/Conjunto de Testes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I101"/>
+  <dimension ref="A1:L101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,6 +460,21 @@
       <c r="I1" t="inlineStr">
         <is>
           <t>acerto_95_fichamento</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>resposta_modelo_rag_fichamento_jev</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>prob_acerto_jev_fichamento_jev</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>acerto_95_fichamento_jev</t>
         </is>
       </c>
     </row>
@@ -547,6 +562,32 @@
       <c r="I2" t="b">
         <v>0</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial [Guia de Orientações sobre Registros 2025.1, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), as atribuições e diferenças de atuação entre o **NAGA**, o **NAREG** e o **NUREC** em relação aos registros acadêmicos e de curso na UFBA são as seguintes:
+*   **NAREG (Núcleo de Admissão e Registros da Graduação):** É responsável por efetuar **registros estudantis** que aparecem no histórico do discente e se aplicam diretamente a ele. Suas atribuições incluem:
+    *   **Admissão de estudantes:** Aluno especial, Aluno Especial - Revalidação, Convênio Instituição Estrangeira (casos raros), Convênio PEC-G, Portador de Diploma (especial), Reingresso imediato, Transferência Interna - especial (3.5.8) e Transferência Ex-Officio;
+    *   Aproveitamento de Estudos e Avaliação de Conhecimento Prévio;
+    *   Cadastro dos discentes (atualização, correção e registro de nome social);
+    *   Cancelamento de matrícula / formas de saída ou inativação (desistência de curso, falecimento, jubilamento por decurso de prazo máximo e recusa de matrícula, mudança de curso e transferência para outra universidade);
+    *   Dilatação de prazo / permanência no curso;
+    *   Semestre de Equivalência;
+    *   Trancamento Parcial e Total.
+*   **NAGA (Núcleo de Apoio e Gestão Acadêmica):** Também atua com **registros estudantis** no histórico do discente, porém voltado a demandas específicas e operacionais de percurso e regularização:
+    *   **Admissão de estudantes:** Cadastro e primeira inscrição em componentes de Alunos de Mobilidade;
+    *   Cumprimento de decisão judicial (via Procuradoria da UFBA — o setor não recebe pedidos diretos de estudantes);
+    *   Inscrição em componentes: Cursos intensivos (já previamente cadastrados pelo NUREC), Estágio e Internato, bem como inscrições fora do prazo (quando houver vagas nas turmas);
+    *   Registro de notas pendentes: Para alunos que solicitaram antecipação de colação de grau, além de notas de estágios, internatos, TCC e monografia.
+*   **NUREC:** Conforme o documento orienta, ao contrário do NAREG e do NAGA (que lidam com registros da vida acadêmica do estudante/histórico), o NUREC é responsável por **registros referentes ao próprio curso** (como, por exemplo, a natureza de um componente curricular), que são efetivados após a conclusão de um processo de alteração curricular. 
+*Vale destacar que nenhum desses três núcleos realiza abertura de processos administrativos; eles atuam exclusivamente executando os registros após a devida tramitação e deliberação.*</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -589,6 +630,18 @@
       </c>
       <c r="I3" t="b">
         <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>De acordo com as diretrizes oficiais da Superintendência de Administração Acadêmica da UFBA, o NAGA (Núcleo de Apoio e Gestão Acadêmica) recebe e processa as demandas de admissão de estudantes por cumprimento de decisão judicial exclusivamente **por meio da Procuradoria UFBA** ([Guia de Orientações sobre Registros Acadêmicos 2025.1, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)). 
+O documento estabelece expressamente que o setor **não recebe pedidos diretos de estudantes** para essa finalidade ([Guia de Orientações sobre Registros Acadêmicos 2025.1, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)). Compete ao NAGA efetuar o registro estudantil correspondente de cadastro e primeira inscrição após a devida tramitação institucional via Procuradoria ([Guia de Orientações sobre Registros Acadêmicos 2025.1, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)).</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L3" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -648,6 +701,26 @@
       <c r="I4" t="b">
         <v>0</v>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>De acordo com as diretrizes do [Guia de Orientações sobre Registros 2025.1 (págs. 1-3)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), os códigos das unidades no sistema SIPAC e os respectivos endereços de e-mail para encaminhamento de demandas são:
+* **NAREG (Núcleo de Admissão e de Registros da Graduação / CARE):**
+  * **Código SIPAC:** `12.01.85.04.01`
+  * **E-mail:** `nareg@ufba.br`
+* **NAGA (Núcleo de Apoio e Gestão Acadêmica / CARE):**
+  * **Código SIPAC:** `12.01.85.04.03`
+  * **E-mail:** `naga@ufba.br`
+* **NARQ (Núcleo de Arquivo / CARE):**
+  * **Código SIPAC:** `12.01.85.04.07`
+  * **E-mail:** `narq@ufba.br`</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -695,6 +768,21 @@
       <c r="I5" t="b">
         <v>0</v>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>De acordo com as orientações oficiais da SUPAC, a classificação e o tratamento de documentos no SIPAC que contêm informações pessoais dos estudantes seguem estas diretrizes:
+* **Classificação como "Restrito":** Os documentos (e não o processo em si) devem ser classificados como **“Restrito”** caso contenham informações pessoais dos estudantes (tais como RG, CPF, endereço, telefone, e-mail, etc.). Mesmo restritos, esses documentos podem ser visualizados normalmente pelas unidades por onde o processo tramita.
+* **Base Legal:** A exigência é fundamentada no **Art. 31 da Lei Federal nº 12.527/2011** (Lei de Acesso à Informação).
+* **Cuidados adicionais (LGPD):** Deve-se evitar a exposição desnecessária de dados pessoais nos documentos cadastrados com a natureza "Ostensivo" (por exemplo, se o nome do aluno já consta no Parecer/Despacho, não é preciso mencionar o número de matrícula no mesmo documento, e vice-versa).
+Essas diretrizes constam na página 1 do [Guia de Orientações sobre Registros 2025.1 (pág. 1)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -736,6 +824,18 @@
         <v>1</v>
       </c>
       <c r="I6" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>De acordo com as orientações do [Guia de Orientações sobre Registros Acadêmicos (SUPAC/CARE)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), pág. 3:
+Em casos excepcionais em que a demanda envolva mais de um estudante como interessado, **o Colegiado (e não o servidor) deve ser cadastrado como interessado** no processo no SIPAC.</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L6" t="b">
         <v>1</v>
       </c>
     </row>
@@ -784,6 +884,20 @@
       <c r="I7" t="b">
         <v>0</v>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial [Guia de Orientações sobre Registros 2025.1, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), caso o equívoco seja de responsabilidade do Colegiado e o processo já se encontre arquivado no Núcleo de Arquivo, o procedimento a ser adotado é o seguinte:
+1. O Colegiado deve solicitar o desarquivamento do processo e o seu envio de volta ao Colegiado por meio de uma mensagem para o e-mail **narq@ufba.br**.
+2. Após o recebimento, deve ser anexado ao processo um despacho informando, de forma objetiva, o que precisa ser corrigido.
+3. Se o caso se tratar de um processo de aproveitamento de estudos, também deverá ser anexada a respectiva **folha de aproveitamento retificada**.</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -825,6 +939,18 @@
       </c>
       <c r="I8" t="b">
         <v>0</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial da Superintendência de Administração Acadêmica (SUPAC), em função da implantação do SIGAA, **não haverá cancelamento de matrícula ou registros de dilatação de prazo/permanência nos semestres 2025.1 e 2025.2**.
+Para mais detalhes e procedimentos institucionais, consulte o [Guia de Orientações sobre Registros 2025.1 da SUPAC/UFBA (pág. 4)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).</t>
+        </is>
+      </c>
+      <c r="K8" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L8" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -890,6 +1016,25 @@
       <c r="I9" t="b">
         <v>0</v>
       </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial [Guia de Orientações sobre Registros 2025.1, pág. 4](https://colest.ime.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), o processo de adoção de nome social por um discente na UFBA possui as seguintes diretrizes:
+* **Documentos de Referência:** Resolução nº 01/2014, de 18/06/14 - CONSEPE, alterada pela Resolução nº 02/2018, de 28/08/18 - CONSEPE.
+* **Fluxo Completo de Tramitação (Procedimento):** O(A) discente solicita a abertura de processo no Núcleo de Atendimento ao Estudante (NAE/SUPAC). O NAE envia o processo à PROGRAD para análise e deliberação e, posteriormente, o processo é encaminhado ao NAREG para a efetivação do registro.
+* **Código CONARQ (SIPAC):** `125.21` - MATRÍCULA. REGISTRO DOS ALUNOS NOS CURSOS DE GRADUAÇÃO (com o assunto detalhado: *Adoção de Nome social*).
+* **Documentação Exigida:** 
+  1. Requerimento preenchido pelo(a) requerente;
+  2. Cópia do documento de identidade;
+  3. Despacho do NAE para a PROGRAD;
+  4. Parecer conclusivo assinado pela PROGRAD.</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -934,6 +1079,21 @@
       </c>
       <c r="I10" t="b">
         <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>De acordo com as normas acadêmicas da UFBA, a apresentação de ementas é exigida nos processos de **Aproveitamento de Estudos** para disciplinas cursadas em **outras Instituições de Ensino Superior (IES)**. 
+Conforme detalhado nos documentos oficiais:
+1. **Art. 10 do Regulamento Acadêmico da Graduação (REGPG):** O aproveitamento de disciplinas cursadas na UFBA ou em outras IES reconhecidas pelo MEC deve ser solicitado junto ao CEAG, sendo instruído obrigatoriamente com o histórico escolar e a ementa oficial (conforme a [Regulamento Acadêmico da Graduação (REGPG/SUPAC), pág. 2](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf)).
+2. **Orientações de Registros Acadêmicos da SUPAC:** A documentação exigida para o processo administrativo especifica a apresentação de *"Ementas das disciplinas (apenas para disciplinas cursadas em outra IES)"*, acompanhada do requerimento, histórico escolar atual e anterior (quando couber) e da Folha de Aproveitamento preenchida (conforme o [Guia de Orientações sobre Registros Acadêmicos 2025.1, pág. 5](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)).
+Portanto, a apresentação das ementas é dispensada apenas para componentes curriculares cursados internamente na própria UFBA, sendo obrigatória para fins de análise de equivalência de conteúdos oriundos de outras faculdades ou universidades externas.</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1003,6 +1163,29 @@
       <c r="I11" t="b">
         <v>0</v>
       </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Com base nos documentos oficiais e regulamentos acadêmicos da UFBA, o procedimento detalhado envolvendo o Colegiado de Curso, o Departamento responsável e o NAREG (Núcleo de Admissão e Registros da Graduação) para a dispensa de componente curricular por meio de **Avaliação de Conhecimento Prévio** ocorre da seguinte forma:
+1. **Solicitação Inicial (Estudante e Colegiado):**
+   - O(A) estudante solicita ao Colegiado de Curso a dispensa de cursar um componente curricular no qual **nunca se inscreveu**, mediante avaliação de conhecimento prévio (conforme a [*Avaliação de Conhecimento Prévio*, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf) do *Guia de Orientações sobre Registros Acadêmicos 2025* e o Artigo 81 do REGPG).
+   - O CCE verifica se o cumprimento do pré-requisito da disciplina está explícito no histórico escolar do solicitante, conforme o [Artigo 1º da Resolução nº 02/2018 do CCE](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf). Além disso, o estudante não pode ter se submetido a exame anteriormente na mesma modalidade com reprovação ou pedido cancelado ([Artigo 2º da Resolução nº 02/2018 do CCE](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf)).
+2. **Deliberação e Encaminhamento pelo Colegiado:**
+   - O Colegiado delibera sobre o pedido (os pedidos recebidos são apreciados na segunda reunião plenária ordinária do CCE de cada semestre, conforme o [Artigo 4º da Resolução nº 02/2018 do CCE](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf)).
+   - Se aprovado, o Colegiado encaminha o processo ao **Departamento responsável** pela disciplina e ao **NAREG** para a devida inscrição provisória no componente (conforme a [*Avaliação de Conhecimento Prévio*, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf) do *Guia de Orientações sobre Registros Acadêmicos 2025*).
+   - A coordenação do CCE informa o estudante sobre o local, data e horário do exame com antecedência mínima de cinco dias úteis, exigindo resposta de ciência em até dois dias úteis ([Artigo 5º da Resolução nº 02/2018 do CCE](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf)).
+3. **Atuação do Departamento:**
+   - O Departamento responsável constitui uma **Comissão de Avaliação**, que realiza o exame, emite um parecer circunstanciado (acompanhado dos exames realizados e do resultado com a nota atribuída, assinado eletronicamente pela Comissão) e envia de volta ao Colegiado (conforme a [*Avaliação de Conhecimento Prévio*, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf) do *Guia de Orientações sobre Registros Acadêmicos 2025*). Ressalta-se que **não há segunda chamada** para este exame, sob hipótese alguma ([Artigo 3º da Resolução nº 02/2018 do CCE](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf)).
+4. **Decisão Final do Colegiado e Registro no NAREG:**
+   - Com base no parecer da Comissão, o Colegiado emite a decisão final por meio de um despacho assinado eletronicamente pelo Coordenador (conforme a [*Avaliação de Conhecimento Prévio*, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf) do *Guia de Orientações sobre Registros Acadêmicos 2025*).
+   - O processo é tramitado e enviado ao **NAREG** (responsável pelos registros estudantis de aproveitamento e dispensa, conforme o [*Guia de Registros*, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf) do *Guia de Orientações sobre Registros Acadêmicos 2025*) para efetivação do registro no histórico escolar do(a) estudante utilizando o código CONARQ `125.23` (Isenção de Disciplinas / Dispensa de Disciplina / Aproveitamento de Estudos com assunto detalhado "Avaliação de conhecimento prévio", conforme a [*Avaliação de Conhecimento Prévio*, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf) do *Guia de Orientações sobre Registros Acadêmicos 2025*).</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1052,6 +1235,22 @@
         <v>0</v>
       </c>
       <c r="I12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial da Superintendência de Administração Acadêmica da UFBA, o cancelamento de matrícula por falecimento de um(a) estudante de graduação (forma de saída/inativação) deve seguir os seguintes procedimentos de comunicação e documentação:
+* **Procedimento de Comunicação:** A ocorrência deve ser informada à SUPAC pelo Colegiado de Curso ou por um familiar. O envio pode ser feito por e-mail diretamente ao Núcleo de Admissão e Registros da Graduação (NAREG) através do endereço `nareg@ufba.br` ou de forma presencial no Núcleo de Atendimento ao Estudante (NAE/SUPAC). Cabe ressaltar que não se aplica código CONARQ específico no SIPAC para este registro.
+* **Documentação Exigida:** 
+  1. **Ofício ou e-mail** enviado pelo Colegiado **acompanhado do atestado de óbito**; **OU**
+  2. **Requerimento escolar** preenchido por algum familiar, **acompanhado do atestado de óbito** e dos **respectivos documentos de identificação** do(a) familiar e do(a) discente.
+Para mais detalhes, consulte o documento [Guia_Orientacoes_Registros_Academicos_2025, pág. 6](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L12" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1121,6 +1320,28 @@
       <c r="I13" t="b">
         <v>0</v>
       </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Com base nos regulamentos e orientações acadêmicas da UFBA, abaixo estão as regras, limitações e procedimentos aplicáveis à inscrição em componentes curriculares fora do prazo, com foco nos casos de **estágio, internato e TCC**:
+### 1. Trabalho de Conclusão de Curso (TCC)
+* **Limitações e Regras:** De acordo com o [Guia de Orientações sobre Registros Acadêmicos 2025.1, p. 7](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), **não há previsão no novo REGPG para inscrição fora do prazo em TCC**. 
+* **Reconhecimento de Carga Horária:** Conforme o Art. 166 do REGPG (citado no [Guia de Orientações sobre Registros Acadêmicos 2025.1, p. 7](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)), caso o discente não esteja devidamente inscrito no componente curricular, a carga horária cursada não será reconhecida pela instituição.
+### 2. Estágio e Internato
+* **Limitações e Regras:** A inscrição fora do prazo é permitida **exclusivamente para componentes de Estágio e Internato**, desde que haja **vagas nas turmas**, conforme estabelecido no [Guia de Orientações sobre Registros Acadêmicos 2025.1, págs. 1 e 6](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).
+* **Procedimento:** O Colegiado do Curso deve enviar um ofício assinado pelo Coordenador para o e-mail do NAGA (`naga@ufba.br`) contendo as seguintes informações e diretrizes:
+  1. Nome completo e número de matrícula do aluno que requisitou a inscrição;
+  2. Código, nome e turma da disciplina;
+  3. Autorização expressa para a liberação de pré-requisito (se for o caso).
+* **Responsabilidade do Colegiado:** É de inteira responsabilidade do Colegiado contatar previamente o(a) professor(a) que ministra a disciplina para alinhar a inscrição ([Guia de Orientações sobre Registros Acadêmicos 2025.1, p. 6](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)).
+* **Documentação necessária:** Um ofício assinado pelo Coordenador do Curso contendo o nome completo do aluno, número de matrícula, código, nome e turma da disciplina ([Guia de Orientações sobre Registros Acadêmicos 2025.1, p. 6](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)).</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L13" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1171,6 +1392,21 @@
         <v>0</v>
       </c>
       <c r="I14" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial da SUPAC, a diferença fundamental reside no fato de que os alunos concluintes de semestres anteriores ao vigente **não podem solicitar o Reingresso Imediato**, sendo permitido a eles apenas a opção de ingresso como **Portador de Diploma - Caráter Especial** (regido pela Seção VI do REGPG) ou a participação em processo seletivo de vagas residuais.
+Abaixo estão detalhadas as características de cada uma das modalidades conforme a documentação:
+*   **Reingresso Imediato:** É uma modalidade restrita e direcionada para permitir ao(a) estudante *concluinte de curso de graduação* o retorno à UFBA em um novo curso **da mesma área básica de ingresso**, observando prazos e documentações específicas (conforme detalhado na seção de Reingresso Imediato da página 1 do guia). Alunos formados em semestres anteriores ao vigente não se enquadram nesta via.
+*   **Portador de Diploma - Caráter Especial:** É a modalidade destinada a permitir que o(a) portador(a) de diploma graduado pela UFBA ingresse em um novo curso de Graduação sem a necessidade de prestar novo vestibular ou ENEM. Esta via é a aplicável aos concluintes de semestres anteriores ao vigente, cujo procedimento é iniciado mediante solicitação ao NAE/SUPAC e posterior avaliação e deliberação do Colegiado do curso (conforme Seção VI do REGPG e as orientações da página 1).
+Para mais detalhes, consulte o documento oficial: [Guia de Orientações sobre Registros Acadêmicos 2025.1, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L14" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1226,6 +1462,26 @@
       </c>
       <c r="I15" t="b">
         <v>0</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>De acordo com as diretrizes do [Guia de Orientações sobre Registros Acadêmicos (pág. 1)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), as informações e os normativos aplicáveis aos pedidos de Reingresso Imediato são os seguintes:
+1. **Informações que devem constar na planilha enviada pelo Colegiado ao NAREG:**
+   A planilha no formato Excel deve conter:
+   - Número de matrícula ou nome completo do discente;
+   - Código do novo curso de ingresso (apenas os números);
+   - Currículo;
+   - Semestre de equivalência.
+   *(Nota: O guia também aponta que é possível anexar as folhas de aproveitamento de estudo).*
+2. **Normativo que rege os pedidos feitos após o prazo do Calendário Acadêmico:**
+   Para os pedidos posteriores ao prazo estabelecido no Calendário Acadêmico, segue-se o disposto na **IN 005/2025 - SUPAC**, conforme explicitado na mesma página do documento.</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -1285,6 +1541,26 @@
       <c r="I16" t="b">
         <v>0</v>
       </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial [Guia de Orientações sobre Registros 2025.1 da SUPAC/UFBA, pág. 8](https://colest.ime.mb.ufba.br/.../Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf) (consulte o documento completo em [Guia de Orientações sobre Registros 2025.1, pág. 8](https://colest.ime.ubfba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)), o procedimento de **Retificação de Saída de Concluinte Jubilado** tem como objetivo regularizar a situação do(a) discente que concluiu o curso, mas teve a matrícula cancelada posteriormente de forma indevida (jubilamento) por ausência de registros ou de tramitação do processo de integralização.
+### Funcionamento do Procedimento
+1. **Avaliação pelo Colegiado:** O Colegiado do curso realiza uma avaliação curricular detalhada. Caso identifique que o(a) estudante concluiu os requisitos do curso antes de ocorrer o jubilamento, o Colegiado preenche e envia uma **ficha de avaliação curricular** por e-mail para o **NIC** (`integralizacao@ufba.br`), com cópia para o **NAREG** (`nareg@ufba.br`) e para o **NAGA** (`naga@ufba.br`), informando o semestre exato da conclusão e justificando a solicitação de retirada do jubilamento e as pendências identificadas.
+### O Papel Específico de Cada Setor na Regularização:
+* **NIC (Núcleo de Integralização Curricular):** 
+  - É o setor responsável por **homologar a conclusão** do curso do(a) discente com base na ficha de avaliação enviada pelo Colegiado.
+* **NAREG (Núcleo de Admissão e Registros da Graduação):** 
+  - Realiza o registro estudantil consistente em **retirar a saída** (o jubilamento indevido) do histórico, além de remover as situações de matrículas posteriores à conclusão (caso tenham ocorrido) conforme detalhado no [Guia de Orientações sobre Registros 2025.1, pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).
+* **NAGA (Núcleo de Apoio e Gestão Acadêmica):** 
+  - Efetua o registro de **resultado pendente de semestres anteriores** (quando aplicável, ressaltando que isso não inclui alteração de registros já existentes na base), conforme estipulado nas diretrizes da SUPAC na [página 8 do Guia de Orientações sobre Registros 2025.1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1335,6 +1611,29 @@
         <v>0</v>
       </c>
       <c r="I17" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Com base nas diretrizes oficiais da UFBA, esclareço os pontos solicitados sobre o **Semestre de Equivalência**:
+### 1. O que é o Semestre de Equivalência?
+Trata-se do semestre letivo a partir do qual se deve começar a computar o tempo despendido pelo(a) aluno(a) de graduação para integralizar o currículo do curso em que está matriculado(a).
+### 2. Como ele deve ser formalizado?
+A indicação do Semestre de Equivalência deve constar de forma expressa:
+* Na **folha de aproveitamento**; OU
+* Por meio de **Ofício** assinado pelo(a) Coordenador(a) do Curso e enviado por e-mail.
+### 3. Qual é o formato padronizado para a sua indicação?
+O formato padronizado obrigatório é composto pelo **ano de ingresso seguido pela indicação do semestre**, utilizando um ponto como separador. 
+* **Exemplo:** `2023.1`
+---
+**Fontes e Referências Oficiais:**
+* As orientações completas sobre o conceito, o documento de referência (Art. 75 do REGPG), o procedimento de formalização e o exemplo de formato estão detalhadas na página 1 do [Guia de Orientações sobre Registros Acadêmicos (SUPAC/CARE)](https://colest.ime.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf).</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L17" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1395,6 +1694,25 @@
         <v>0</v>
       </c>
       <c r="I18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Com base no [Guia de Orientações sobre Registros Acadêmicos (pág. 9)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), as duas formas/modalidades de solicitação de trancamento (parcial e total) e os respectivos procedimentos e códigos CONARQ correspondentes são:
+1. **Trancamento Parcial (de disciplina/componente curricular):**
+   * **Procedimento 1:** Realizado diretamente pelo(a) estudante por meio do sistema acadêmico (SIGAA) no período estabelecido no Calendário Acadêmico.
+   * **Procedimento 2 / Excepcional:** Apresentação de pedido de trancamento a qualquer tempo dentro do semestre, com devida justificativa e documentos comprobatórios, direcionado ao NAE/SUPAC ou ao Colegiado.
+   * **Código CONARQ (SIPAC):** **125.241** (Trancamento de Disciplina / Trancamento Parcial de Curso).
+2. **Trancamento Total (de matrícula/curso):**
+   * **Procedimento 1:** Realizado pelo(a) estudante por meio do sistema acadêmico no período estabelecido no Calendário Acadêmico (a STI processa as solicitações).
+   * **Procedimento 2 / Excepcional:** Apresentação de pedido de trancamento a qualquer tempo dentro do semestre, com justificativa e documentos comprobatórios (como relatório médico, se por motivo de saúde), junto ao NAE/SUPAC ou ao Colegiado.
+   * **Código CONARQ (SIPAC):** **125.242** (Trancamento Total de Curso / Matrícula Total).</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L18" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1450,6 +1768,19 @@
       <c r="I19" t="b">
         <v>0</v>
       </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>De acordo com o documento oficial [Guia de Orientações sobre Registros Acadêmicos (SUPAC/CARE)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf):
+* **Cursos contemplados:** A modalidade de **Transferência Interna - Especial** é destinada a discentes regulares de cursos de graduação integrados a uma **mesma área básica de ingresso**, além dos cursos da **Escola de Música**, da **Escola de Teatro** e de **Letras** (conforme descrito na página 9/10 do guia).
+* **Restrições aplicáveis (como no caso da Escola de Música):** A transferência interna especial **não** pode ser feita para qualquer curso da UFBA de forma livre. O guia estabelece explicitamente que **um(a) estudante da Escola de Música só pode ser transferido(a) para outro curso da própria Escola de Música**. Caso o(a) discente deseje mudar para um curso fora da sua área básica de ingresso ou de sua unidade (como mudar da Escola de Música para outro curso), a mudança não ocorre por transferência especial, sendo obrigatória a participação no **processo seletivo de Vagas Residuais** (conforme detalhado na página 10).</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L19" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1505,6 +1836,28 @@
       <c r="I20" t="b">
         <v>0</v>
       </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>De acordo com a **Instrução Normativa nº 006/2025 da SUPAC/UFBA**, as regras referentes ao envio e aos dados da lista única de solicitações de trancamento de TCC são as seguintes:
+### 1. Prazo Limite
+O Colegiado deverá julgar as solicitações de trancamento e encaminhar a lista única ao setor de registros **até o último dia de lançamento de notas e conceitos**, conforme definido no calendário acadêmico (*Art. 2º*, págs. 1-2). 
+* **Forma de envio:** A lista, datada e assinada pela Coordenação do Curso, deve ser enviada para o e-mail **nareg@ufba.br** com o assunto: `Trancamento de TCC` (*Art. 2º, Inciso I*, pág. 2).
+* **Atenção:** Solicitações enviadas após o último dia de lançamento de notas não serão registradas (*Art. 3º*, pág. 2).
+### 2. Dados Obrigatórios na Lista
+Conforme o *Art. 2º, Inciso II* (pág. 2), a lista deve conter obrigatoriamente as seguintes informações:
+* Nome completo do(a) estudante;
+* Número de matrícula;
+* Código do componente curricular referente ao TCC;
+* Nome do componente curricular referente ao TCC.
+Você pode consultar o teor completo e os detalhes normativos no documento oficial por meio do link: [Instrução Normativa nº 006/2025, págs. 1-2](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Instrucao_Normativa_N%C2%BA_006_2025.pdf).</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L20" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1556,6 +1909,22 @@
       <c r="I21" t="b">
         <v>0</v>
       </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>De acordo com o **Parágrafo único do Art. 3º da Instrução Normativa nº 006/2025 da SUPAC**, em situação extraordinária de perda do prazo pelo Colegiado no envio da lista única, a autorização de trancamento de TCC deverá ser tramitada por meio de **processo administrativo** cadastrado no SIPAC sob o código **125.241** com o assunto **"Trancamento de TCC"**.
+Para isso, o processo deverá conter os seguintes documentos anexados:
+1. A **ata** com a decisão da plenária do Colegiado sobre o(s) trancamento(s) solicitado(s);
+2. A **anuência** do(s) docente(s) orientador(es);
+3. O(s) **requerimento(s)** de solicitação apresentado(s) pelo(s) estudante(s).
+Mais detalhes podem ser consultados diretamente no documento oficial: [Instrução Normativa nº 006/2025, págs. 1-2](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Instrucao_Normativa_N%C2%BA_006_2025.pdf).</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L21" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1604,6 +1973,23 @@
       <c r="I22" t="b">
         <v>0</v>
       </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>De acordo com a **Instrução Normativa nº 006/2025 da SUPAC/UFBA** e o **Regulamento de Ensino de Graduação e Pós-Graduação (REGPG)**, as restrições temporais e de histórico escolar que impedem o pedido ou o registro do trancamento de TCC são as seguintes:
+### Restrições Temporais e de Prazos:
+1. **Prazo Semestral Obrigatório:** Em atenção ao art. 54 do REGPG, o pedido de trancamento de TCC deve ocorrer obrigatoriamente no semestre objeto da solicitação, sendo **vetado** ao Colegiado receber pedidos fora desse prazo (*Art. 1º, § 1º da [Instrução Normativa nº 006/2025, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Instrucao_Normativa_N%C2%BA_006_2025.pdf)*).
+2. **Proibição de Retroatividade:** A solicitação de trancamento **não pode alcançar semestres pretéritos**, conforme o disposto no artigo 64 do REGPG (*Art. 1º, § 2º da [Instrução Normativa nº 006/2025, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Instrucao_Normativa_N%C2%BA_006_2025.pdf)*).
+3. **Prazo de Envio pela Coordenação:** Solicitações de trancamento de TCC enviadas pelo Colegiado para registro após o último dia de lançamento de notas estabelecido no calendário acadêmico **não serão registradas** (*Art. 3º da [Instrução Normativa nº 006/2025, pág. 2](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Instrucao_Normativa_N%C2%BA_006_2025.pdf)*).
+### Restrições de Histórico Escolar:
+1. **Existência de Conceito Registrado:** O trancamento **não será registrado** nos casos em que o(a) discente já possua resultado ou conceito (aprovado ou reprovado) lançado e registrado no histórico escolar (*Art. 4º da [Instrução Normativa nº 006/2025, pág. 2](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Instrucao_Normativa_N%C2%BA_006_2025.pdf)*).</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L22" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1650,6 +2036,22 @@
         <v>0</v>
       </c>
       <c r="I23" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Com base no **Projeto Pedagógico e Diretrizes do Curso de Bacharelado em Estatística da Universidade Federal da Bahia (UFBA)** ([Projeto_Pedagogico_Estatistica_Bacharelado, págs. 1-2](https://colest.ime.ufba.br/)), as informações oficiais sobre o curso são as seguintes:
+* **Número de vagas anuais:** O curso oferece anualmente **60 (sessenta) vagas**, com ingresso no primeiro semestre letivo por meio do Sistema de Seleção Unificada (SiSU/ENEM), conforme o § 1º do Art. 1º.
+* **Turno preferencial:** As componentes curriculares são ministradas preferencialmente no **turno matutino**, conforme o § 2º do Art. 1º.
+* **Prazos de integralização:** 
+  * **Prazo médio (duração):** **8 (oito) semestres**, de acordo com o § 2º do Art. 1º.
+  * **Prazo máximo:** **16 (dezesseis) semestres**, conforme o § 2º do Art. 1º.</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L23" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1705,6 +2107,32 @@
         <v>0</v>
       </c>
       <c r="I24" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>De acordo com os documentos oficiais do curso de Bacharelado em Estatística da UFBA, os requisitos de carga horária prévia e de composição da banca examinadora para o Trabalho de Conclusão de Curso (TCC) são os seguintes:
+### 1. Requisitos de Carga Horária para Início
+* **Submissão do Projeto:** O(a) discente deve submeter o projeto de TCC ao Colegiado após ter integralizado, no mínimo, **75% da carga horária obrigatória** do curso.
+* **Desenvolvimento:** O TCC é desenvolvido ao longo de duas disciplinas obrigatórias: MATD52 (Trabalho de Conclusão de Curso I - TCCI) e MATD53 (Trabalho de Conclusão de Curso II - TCCII).
+*Fontes:* 
+* Art. 4º, § 1º do [Projeto Pedagógico e Diretrizes do Curso de Bacharelado em Estatística da UFBA, pág. 1](https://colest.ime.ufba.br/).
+* [Resolução nº 05/2024 - Colegiado do Curso de Estatística, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).
+---
+### 2. Requisitos da Banca Examinadora
+* **Composição:** A banca examinadora do TCCI e do TCCII deve ser composta obrigatoriamente por **3 (três) membros titulares**, indicados pelo professor orientador.
+* **Critérios de Formação:** 
+  1. No mínimo **dois professores membros do Departamento de Estatística da UFBA**, o que já inclui o próprio orientador.
+  2. Na existência concomitante de orientador e coorientador, **apenas um deles** poderá compor a banca examinadora.
+*Fontes:* 
+* Art. 4º, § 2º do [Projeto Pedagógico e Diretrizes do Curso de Bacharelado em Estatística da UFBA, pág. 1](https://colest.ime.ufba.br/).
+* Art. 7º e parágrafo único da [Resolução nº 05/2024 - Colegiado do Curso de Estatística, pág. 2](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L24" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1781,6 +2209,32 @@
       <c r="I25" t="b">
         <v>0</v>
       </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Com base nos regulamentos acadêmicos oficiais da UFBA e do curso de Bacharelado em Estatística, seguem as diretrizes referentes ao **trancamento total de matrícula** e às situações de **desligamento por jubilamento**:
+---
+### 1. Regras para o Trancamento Total de Matrícula
+O trancamento total consiste na suspensão temporária de todas as atividades acadêmicas do discente no semestre letivo corrente. As normas gerais e específicas estabelecem que:
+* **Limite de tempo:** O trancamento total pode ser concedido por **até 4 (quatro) semestres letivos** ao longo de todo o curso, podendo ser consecutivos ou intercalados (conforme o [Regulamento Acadêmico da Graduação (REGPG), Art. 4º, § 1º, pág. 1](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf) e o [Projeto Pedagógico do Curso de Estatística, Art. 5º, § 2º, pág. 1](https://colest.ime.ufba.br/)).
+* **Contagem de prazo:** Os períodos de trancamento total **não** são computados para o cálculo do prazo máximo de integralização curricular, nem permitem a realização de estágios durante o período de suspensão (conforme o [REGPG, Art. 4º, § 2º, pág. 1](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf) e o [Projeto Pedagógico do Curso de Estatística, Art. 5º, § 2º, pág. 1](https://colest.ime.ufba.br/)).
+* **Restrição para calouros:** O trancamento total **não é permitido** no primeiro semestre letivo de ingresso do estudante na UFBA (semestre de calouro), **salvo** por motivo de doença grave devidamente comprovada por junta médica oficial da UFBA ou por prestação de serviço militar obrigatório (conforme o [REGPG, Art. 4º, § 3º, pág. 1](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf)).
+* **Trancamento por motivo de saúde:** Pode ser requerido a qualquer momento do semestre letivo, mediante abertura de processo no CEAG instruído com laudo médico homologado pelo SMURB/UFBA (conforme o [REGPG, Art. 5º, pág. 1](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf)).
+* **Prazos e Solicitação:** Alunos veteranos realizam o pedido via sistema informatizado (SIGAA) dentro do prazo do Calendário Acadêmico. Solicitações fora do prazo (intempestivas) e pedidos de trancamento total ou parcial por motivos relevantes específicos (como problemas de saúde, óbito de parente próximo, maternidade ou alteração na jornada de trabalho) seguem as diretrizes detalhadas na [Resolução Nº 01/2018 do Colegiado de Estatística, Art. 3º e 4º, págs. 1-2](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf).
+---
+### 2. Situações que Configuram o Desligamento por Jubilamento (Cancelamento do Registro Acadêmico)
+O cancelamento do registro acadêmico e o desligamento do discente ocorrem nas seguintes situações previstas institucionalmente:
+* **Esgotamento de prazo:** Quando o estudante esgotar o prazo máximo de integralização curricular do curso — que para o Bacharelado em Estatística é de **16 (dezesseis) semestres** — acrescido das eventuais dilatações de prazo concedidas (conforme o [REGPG, Art. 9º, § 1º, pág. 2](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf) e o [Projeto Pedagógico do Curso de Estatística, Art. 1º, § 2º e Art. 5º, § 3º, págs. 1-2](https://colest.ime.ufba.br/)).
+* **Reprovação por falta consecutiva:** Quando o discente for reprovado por falta (RF) em **todas** as disciplinas em que estiver matriculado por **2 (dois) semestres consecutivos** (conforme o [REGPG, Art. 9º, § 2º, pág. 2](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf) e o [Projeto Pedagógico do Curso de Estatística, Art. 5º, § 3º, págs. 1-2](https://colest.ime.ufba.br/)).
+* **Abandono de curso:** Quando o estudante deixar de realizar a matrícula ou o trancamento em semestre letivo regular (conforme o [REGPG, Art. 9º, § 3º, pág. 2](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf)).
+* **Reprovação reincidente em disciplina obrigatória:** Quando o discente for reprovado por **4 (quatro) vezes** na mesma disciplina obrigatória, ressalvado o plano especial de acompanhamento concedido pelo Colegiado (conforme o [REGPG, Art. 9º, § 4º, pág. 2](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf)).</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="L25" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1835,6 +2289,27 @@
         <v>0</v>
       </c>
       <c r="I26" t="b">
+        <v>0</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Com base no [Regulamento Acadêmico da Graduação (REGPG/SUPAC)](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf) da UFBA, seguem as orientações referentes à carga horária mínima semestral e ao trancamento parcial de disciplinas:
+### 1. Carga Horária Mínima Semestral (Matrícula Regular)
+* De acordo com o **Art. 2º** do [Regulamento Acadêmico da Graduação (REGPG/SUPAC), pág. 1](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf), a carga horária semestral máxima e mínima permitida obedece aos limites previstos no Projeto Pedagógico de cada Curso (PPC). 
+* A carga horária **não pode ser inferior a 3 (três) componentes curriculares ou ao equivalente a 180 horas semestrais**, ressalvados os períodos finais de integralização.
+---
+### 2. Restrições Aplicáveis ao Trancamento Parcial de Disciplinas
+Conforme o **Art. 3º** do [Regulamento Acadêmico da Graduação (REGPG/SUPAC), pág. 1](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf) e as diretrizes do Colegiado ([Resolução nº 01/2018 do Colegiado de Estatística](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf)), as principais restrições e regras são:
+* **Prazo:** O trancamento parcial deve ser solicitado por meio do SIGAA até o limite de data fixado no Calendário Acadêmico oficial da UFBA (**§ 1º do Art. 3º do REGPG**).
+* **Limite Mínimo de Carga Horária:** **Não é permitido** o trancamento parcial quando este resultar em uma carga horária ou número de disciplinas inferior ao limite mínimo semestral estabelecido pelo Colegiado (**§ 2º do Art. 3º do REGPG**).
+* **Repetição:** É **vedado** o trancamento parcial de uma mesma disciplina por **mais de duas vezes consecutivas** (**§ 3º do Art. 3º do REGPG**).
+* **Indeferimentos pelo Colegiado:** Solicitações de trancamento iniciadas fora do prazo ou que se enquadrem em situações como conflito com horários de estágio, trabalho (cuja admissão/mudança tenha ocorrido antes do período de matrícula), falta de comprovação médica ou dedicação a atividades extracurriculares (como monitoria e iniciação científica) serão **indeferidas**, conforme detalha o **Art. 4º** da [Resolução nº 01/2018 do Colegiado de Estatística, pág. 2](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf).</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="L26" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1895,6 +2370,27 @@
       <c r="I27" t="b">
         <v>0</v>
       </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>De acordo com as normas acadêmicas da UFBA, as regras sobre o trancamento total de matrícula no primeiro semestre letivo (período de calouro) e o procedimento por motivo de saúde estabelecem o seguinte:
+### 1. Situações em que o estudante calouro pode solicitar o trancamento total
+Em regra, o trancamento total não é permitido no primeiro semestre letivo de ingresso do estudante na UFBA (**semestre de calouro**). No entanto, conforme o **§ 3º do Art. 4º do Capítulo II do [Regulamento Acadêmico da Graduação (REGPG/SUPAC)](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf)** (pág. 1), o estudante calouro **pode** solicitar e ter o trancamento total deferido exclusivamente em duas situações de exceção:
+* Por motivo de **doença grave** devidamente comprovada por junta médica oficial da UFBA;
+* Por motivo de **prestação de serviço militar obrigatório**.
+Adicionalmente, a **[Resolução nº 01/2018 do Colegiado de Estatística](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf)** (págs. 1-2) prevê no **Art. 3º, inciso II** que as solicitações de trancamento total por parte de alunos ingressantes devem ser requeridas via processo dentro do período estabelecido na agenda acadêmica da UFBA (já que para os calouros não é permitida a solicitação direta pelo sistema informatizado).
+### 2. Como funciona o pedido por motivo de saúde
+Conforme o **Art. 5º do Capítulo II do [Regulamento Acadêmico da Graduação (REGPG/SUPAC)](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf)** (pág. 1) e o detalhamento do **[Guia de Orientações sobre Registros Acadêmicos (SUPAC/CARE)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf)** (pág. 9):
+* O trancamento total por motivos de saúde (trancamento com justificativa médica) **pode ser requerido a qualquer tempo** durante o semestre letivo.
+* O procedimento exige a abertura de um processo no **CEAG** (ou apresentação ao NAE/SUPAC / Colegiado).
+* O pedido deve ser devidamente instruído com **laudo médico homologado pelo SMURB/UFBA** (ou relatório médico, conforme os documentos comprobatórios exigidos para o código CONARQ 125.242 de trancamento total por motivo de saúde).</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="L27" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1948,6 +2444,29 @@
         <v>0</v>
       </c>
       <c r="I28" t="b">
+        <v>0</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Com base no [Regulamento Acadêmico da Graduação (REGPG / SUPAC)](https://supac.ufba.br/sites/supac.ufba.br/files/guia_do_estudante_supac.pdf) da UFBA, seguem as orientações detalhadas para cada um dos pontos solicitados:
+### 1. Critérios de Nota e Frequência para Aprovação
+* **Notas:** O aproveitamento em cada componente curricular é expresso por notas de 0 (zero) a 10 (dez). Para ser considerado aprovado, o discente deve obter nota final **igual ou superior a 5,0 (cinco vírgula zero)** (*Art. 6º, pág. 1*).
+* **Frequência:** A frequência mínima exigida é de **75% (setenta e cinco por cento)** da carga horária ministrada. O aluno com frequência inferior a 75% será reprovado por falta (RF), independentemente da média de notas obtida (*Art. 6º, § 1º, pág. 1*).
+---
+### 2. Prazos para Segunda Chamada e Revisão de Nota
+* **Segunda Chamada:** O aluno que deixar de comparecer a uma avaliação por **motivo justificado** (doença, luto de primeiro grau ou convocação judicial) poderá requerer a 2ª chamada no prazo de **até 72 (setenta e duas) horas** após a realização da prova, junto ao CEAG/Colegiado (*Art. 6º, § 2º, pág. 1*).
+* **Revisão de Nota / Recorreção de Prova:** O estudante tem direito de vista de prova e de solicitar recorreção ou revisão de nota no prazo de **até 5 (cinco) dias úteis** após a divulgação oficial do resultado pelo docente (*Art. 7º, pág. 1*).
+---
+### 3. Exigência Mínima de Compatibilidade para Aproveitamento de Estudos
+* **Aproveitamento de Disciplinas:** O aproveitamento de disciplinas cursadas na UFBA ou em outras Instituições de Ensino Superior (IES) reconhecidas pelo MEC é solicitado junto ao CEAG, mediante ementa oficial e histórico escolar (*Art. 10, pág. 2*). A equivalência exige uma **compatibilidade mínima de 80% (oitenta por cento)** do conteúdo programático e carga horária equivalente (*Art. 10, § 1º, pág. 2*).
+---
+Se precisar de mais detalhes sobre prazos no SIGAA ou procedimentos específicos do curso de Estatística, estou à disposição!</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L28" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2005,6 +2524,20 @@
       <c r="I29" t="b">
         <v>0</v>
       </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>De acordo com a **Resolução nº 01/2018 do Colegiado de Estatística da UFBA**, a diferença de procedimento entre alunos veteranos e ingressantes para solicitar o trancamento total ou parcial dentro do período estabelecido na agenda acadêmica é a seguinte:
+* **Alunos Veteranos:** Devem realizar a solicitação diretamente **via sistema informatizado de registro e controle acadêmico institucional** (em conformidade com o Artigo 67 do REGPG), dentro do prazo estipulado na agenda acadêmica da UFBA (Art. 3º, Inciso I).
+* **Alunos Ingressantes:** Devem realizar a solicitação **via processo**, dentro do período estabelecido na agenda acadêmica da UFBA. Para os alunos ingressantes, **não é permitida** a solicitação por meio do sistema informatizado de registro e controle acadêmico institucional (Art. 3º, Inciso II).
+Você pode consultar os detalhes na íntegra no documento [Resolução nº 01/2018 do Colegiado de Estatística, pág. 1](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf).</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L29" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2059,6 +2592,24 @@
       <c r="I30" t="b">
         <v>0</v>
       </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>De acordo com a **[Resolução nº 01/2018 do Colegiado de Estatística da UFBA](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf)** (págs. 1-2), os pedidos de trancamento total ou parcial iniciados **fora do período** estabelecido na agenda acadêmica (em casos de intempestividade) e que possuem um **motivo relevante ocorrido após o prazo** terão seus pedidos deferidos quando se enquadrarem nas seguintes situações previstas no Artigo 3º, Inciso III:
+* **a)** Atipicidade do semestre, quando definida pelo Conselho Superior de Ensino, Pesquisa e Extensão da UFBA (por exemplo, greve);
+* **b)** Problema de saúde relevante do próprio requerente, desde que comprovado por atestado ou relatório médico, levando em consideração as informações constantes no documento;
+* **c)** Problema de saúde relevante de parente próximo (pai, mãe, irmãos, filhos, cônjuge ou outros que tenham papel similar na vida do aluno), desde que comprovado por relatório médico e suas respectivas informações;
+* **d)** Óbito de parente próximo (pai, mãe, irmãos, filhos, cônjuge ou outros com papel similar na vida do aluno), atestado por meio de documento de óbito;
+* **e)** Maternidade a menos de quatro meses, desde que apresentada certidão de nascimento ou documento de adoção;
+* **f)** Necessidade de trabalho, desde que a admissão ou mudança de jornada tenha acontecido **após** o período de matrícula e esteja devidamente documentada pela empresa.
+Ademais, o Artigo 4º da mesma resolução destaca que solicitações fora do prazo serão explicitamente **indeferidas** caso ocorram por motivos como matrícula em outro curso superior, conflito com horário de estágio, conflito com horário de trabalho (quando a admissão/mudança ocorreu *antes* do período de inscrição), problemas de saúde sem comprovação médica, dedicação a atividades extracurriculares (iniciação científica, monitorias, etc.) ou quaisquer outros motivos sem documentação comprobatória ou ocorridos antes do período de inscrições.</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L30" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2102,6 +2653,19 @@
         <v>0</v>
       </c>
       <c r="I31" t="b">
+        <v>0</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Com base na [Resolução nº 01/2018 do Colegiado de Estatística da UFBA](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.p), as condições relacionadas ao conflito de horário de trabalho que levam ao deferimento ou indeferimento de um pedido de trancamento fora do prazo (iniciado após o período estabelecido na agenda acadêmica) são as seguintes:
+* **Deferimento (Art. 3º, alínea "f", pág. 2):** O pedido será deferido por motivo de **necessidade de trabalho**, desde que a admissão ou a mudança de jornada tenha acontecido **após o período de matrícula** e esteja devidamente documentada pela empresa.
+* **Indeferimento (Art. 4º, inciso III, pág. 2):** O pedido será indeferido se o conflito com o horário de trabalho ocorrer quando a admissão ou a mudança de jornada tiver acontecido **antes do período de inscrição em componentes curriculares**.</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L31" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2155,6 +2719,24 @@
       <c r="I32" t="b">
         <v>0</v>
       </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 4º da Resolução nº 01/2018 do Colegiado de Estatística da UFBA**, as solicitações de trancamento total ou parcial de inscrição em componentes curriculares terão seus pedidos **indeferidos** quando os processos forem iniciados fora do período estabelecido na agenda acadêmica da UFBA nas seguintes situações:
+I - por matrícula em outro curso superior;  
+II - por motivo de conflito com horário de estágio;  
+III - por motivo de conflito com horário de trabalho, desde que a admissão ou mudança de jornada tenha acontecido antes do período de inscrição em componentes curriculares;  
+IV - por problemas de saúde não comprovados com atestado ou relatório médico;  
+V - dedicação a atividades extracurriculares, tais como, projetos de iniciação científica, monitorias, etc., pelo entendimento de que a participação em tais atividades não deve prejudicar o desempenho do aluno no curso;  
+VI - por outro qualquer motivo sem documentação comprobatória ou ocorrido anteriormente ao período de inscrição em componentes curriculares.
+Para mais detalhes, consulte o documento oficial: [Resolução nº 01/2018, págs. 1-2](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf).</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L32" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2197,6 +2779,21 @@
       </c>
       <c r="I33" t="b">
         <v>1</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 6º da Resolução nº 01/2018** do Colegiado de Estatística da UFBA, a solicitação de permanência no curso de Bacharelado em Estatística será deferida, mediante a comprovação da justificativa, quando ocorrer uma das seguintes situações:
+1. **Tratar-se do primeiro pedido de permanência** do aluno que tenha integralizado, no mínimo, **80% da carga horária total do curso** (Inciso I).
+2. O pedido for motivado **por motivo de saúde**, devidamente comprovado com **relatório médico** (Inciso II).
+Conforme estipulado no **Art. 7º** da mesma norma, eventuais casos omissos devem ser julgados diretamente pelo Colegiado do Curso de Estatística.
+Você pode consultar o documento completo por meio do seguinte link: [Resolução nº 01/2018 - Trancamento e Permanência, pág. 3](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-01_2018_Trancamento-e-Perman%C3%AAncia.pdf).</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L33" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -2242,6 +2839,22 @@
         <v>0</v>
       </c>
       <c r="I34" t="b">
+        <v>0</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>De acordo com a regulamentação do curso de Bacharelado em Estatística da UFBA, **é expressamente vetado o pedido de avaliação de conhecimento prévio para os Trabalhos de Conclusão de Curso (TCC)**, mesmo que o discente seja provável concluinte.
+Essa determinação está estabelecida no **Artigo 8º da [Resolução nº 02/2018 do Colegiado de Estatística](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf)** (págs. 1-2):
+&gt; *"Art. 8º É vetado o pedido de avaliação de conhecimento prévio de trabalhos de conclusão de curso, ainda que para aluno concluinte;"*
+Além disso, a mesma resolução aponta outras vedações gerais que impedem que determinado componente curricular seja objeto desse tipo de avaliação (Art. 2º):
+* Componentes nos quais o aluno já tenha se submetido a exame anteriormente na mesma modalidade e tenha sido **reprovado**; ou
+* Componentes cujos pedidos anteriores tenham sido **cancelados** (conforme o Art. 5º da referida norma).</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="L34" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2295,6 +2908,23 @@
         <v>0</v>
       </c>
       <c r="I35" t="b">
+        <v>0</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Com base na [Resolução nº 02/2018 do Colegiado de Estatística da UFBA (CCE)](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf), que delibera sobre a dispensa de cursar componente curricular mediante avaliação de conhecimento prévio, seguem as diretrizes e prazos referentes à comunicação, ciência e faltas:
+1. **Prazos de Comunicação e Confirmação de Ciência:**
+   - De acordo com o **Art. 5º** (págs. 1-2), o solicitante deve ser informado pela coordenação do CCE, com uma **antecedência mínima de cinco dias úteis**, sobre o local, data e horário da aplicação do exame.
+   - O(a) estudante deve responder à mensagem eletrônica enviada pelo CCE dando ciência dessas informações no **prazo de dois dias úteis** (alínea *a* do Art. 5º, pág. 2). Caso as informações sejam passadas pessoalmente, a ciência deve ser feita por escrito e assinada por ambas as partes (alínea *b* do Art. 5º, pág. 2).
+2. **O que ocorre caso o estudante não confirme ciência ou falte:**
+   - **Falta de confirmação:** Conforme a alínea *a* do **Art. 5º** (pág. 2), se o estudante não responder à mensagem eletrônica dando ciência no prazo de dois dias úteis, terá **seu pedido cancelado**.
+   - **Falta à prova (Segunda chamada):** O **Art. 3º** da resolução estabelece expressamente que **está vetada a segunda chamada** do exame de avaliação de conhecimento prévio sob qualquer hipótese (pág. 1).</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L35" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2365,6 +2995,20 @@
       <c r="I36" t="b">
         <v>0</v>
       </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>De acordo com a **Resolução nº 02/2018** do Colegiado de Estatística da UFBA, as regras sobre o limite de solicitações, instrução dos processos e apreciação das avaliações de conhecimento prévio são as seguintes:
+* **Limite de solicitações:** O Art. 7º estabelece que o limite será de, **no máximo, dois pedidos por aluno em cada semestre letivo**. Caso o estudante envie um número superior, caberá a ele o direito de escolher quais dois processos serão encaminhados às instâncias pertinentes (pág. 2). Além disso, o Art. 8º veda totalmente pedidos para trabalhos de conclusão de curso (pág. 2).
+* **Instrução dos processos:** Conforme o Art. 6º, havendo mais de um pedido de avaliação de conhecimento prévio de um mesmo aluno, **estes devem ser instruídos em processos separados** (pág. 2). Adicionalmente, de acordo com as diretrizes de documentação da [Guia de Orientações sobre Registros Acadêmicos 2025 (pág. 1)](https://colest.ime.ufba.br/wp-content/uploads/2025/04/Guia-de-Orienta%C3%A7%C3%B5es-sobre-Registros-2025.1.pdf), o processo deve conter o requerimento do estudante, o pedido de inscrição no componente, relatório circunstanciado com os exames realizados e a devida avaliação com indicação da nota (assinada eletronicamente pela Comissão de Avaliação), além do despacho do Colegiado com a decisão final.
+* **Apreciação pelo Colegiado:** O Art. 4º da [Resolução nº 02/2018 (pág. 1)](http://colest.ime.ufba.br/wp-content/uploads/2019/03/Resolu%C3%A7%C3%A3o-02_2018_Exame_Conhecimento_Previo.pdf) determina que os pedidos recebidos **somente serão apreciados na segunda reunião plenária ordinária do CCE de cada semestre letivo**.</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L36" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2411,6 +3055,20 @@
         <v>1</v>
       </c>
       <c r="I37" t="b">
+        <v>1</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>De acordo com os documentos oficiais do Colegiado do Curso de Bacharelado em Estatística da UFBA:
+* **Carga horária total do curso:** A formação para a obtenção do título de Bacharel em Estatística consiste em uma carga horária total de **3.000 horas** (conforme o *Art. 1º da [Resolução nº 03/2025, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)*).
+* **Atividades Complementares (AC):** O discente deve perfazer uma carga horária mínima de **150 horas** obrigatórias de Atividades Complementares para a integralização da grade curricular de 2023.1 (*Art. 1º da [Resolução nº 03/2025, pág. 1](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)*).
+* **Atividades Extensionistas:** Para os ingressantes a partir de 2023.1, estabelece-se que uma carga horária mínima de **120 horas** (das 150 horas totais obrigatórias de Atividade Complementar) deverá ser caracterizada especificamente como Atividade Extensionista (*Art. 4º da [Resolução nº 03/2025, pág. 2](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)*).</t>
+        </is>
+      </c>
+      <c r="K37" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L37" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2474,6 +3132,32 @@
       <c r="I38" t="b">
         <v>0</v>
       </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Com base na **Resolução nº 03/2025** do Colegiado do Curso de Bacharelado em Estatística da UFBA, as condições temporais e documentais para o aproveitamento de horas de Atividades Complementares (AC) anteriores à matrícula atual, aplicáveis a discentes reingressantes ou com transferência *ex officio*, são as seguintes:
+### 1. Condições Temporais
+* **Prazo limite:** As atividades devem ter sido realizadas há, no máximo, **três anos** antes da data da matrícula atual (conforme o § 1º do Art. 2º).
+* **Origem:** Podem ser horas desenvolvidas tanto na própria UFBA quanto em outra instituição de ensino superior (IES) em período anterior ao reingresso ou à transferência *ex officio* (conforme o § 1º do Art. 2º).
+### 2. Condições Documentais
+* **Forma de comprovação:** 
+  * Para **reingressantes**: A carga horária deve estar devidamente comprovada no **histórico escolar** (conforme o § 2º do Art. 2º).
+  * Para **transferência *ex officio***: A comprovação deve ser feita por meio de **documentação oficial da instituição de ensino superior** de origem (conforme o § 2º do Art. 2º).
+* **Requisitos gerais dos comprovantes (§ 4º do Art. 5º):** Os documentos apresentados devem conter obrigatoriamente:
+  * Nome completo do discente;
+  * Timbre da instituição que forneceu o documento;
+  * Assinatura do responsável pela instituição ou pela atividade;
+  * Descrição das atividades desenvolvidas pelo discente;
+  * Data de início e término;
+  * Carga horária total.
+Para mais detalhes, consulte o documento oficial: [Resolução nº 03/2025 - Atividades Complementares do Curso de Estatística, págs. 1-2](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf).</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L38" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2518,6 +3202,21 @@
         <v>1</v>
       </c>
       <c r="I39" t="b">
+        <v>0</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>De acordo com a regulamentação do curso de Bacharelado em Estatística da UFBA, os prazos e a frequência para a entrega dos documentos comprobatórios das Atividades Complementares (AC) são os seguintes:
+1. **Prazo Limite:** 
+   Conforme o **Art. 5º da [Resolução nº 03/2025 do Colegiado do Curso de Estatística (pág. 2)](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)**, a entrega dos documentos comprobatórios deve ocorrer **no máximo até o penúltimo semestre previsto para conclusão de curso**, garantindo que o procedimento seja realizado em tempo hábil para a avaliação curricular e a consequente diplomação dos prováveis concluintes.
+2. **Frequência de Entrega:** 
+   De acordo com o **§ 1º do Art. 5º da [mesma resolução (pág. 2)](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)**, o(a) discente deverá entregar os documentos para integralizar a carga horária de atividade complementar **uma única vez ao longo do curso**, assim que tiver alcançado a carga horária total exigida (mínimo de 150 horas, observando os limites por modalidade descritos no Anexo 1).</t>
+        </is>
+      </c>
+      <c r="K39" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L39" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2578,6 +3277,23 @@
       <c r="I40" t="b">
         <v>0</v>
       </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>De acordo com o **§ 4º do Art. 5º** da [Resolução Nº 03/2025 do Colegiado do Curso de Bacharelado em Estatística da UFBA](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf) (págs. 2-3), os documentos comprobatórios de Atividades Complementares anexados no sistema acadêmico devem conter obrigatoriamente as seguintes informações:
+1. **Nome completo do discente**;
+2. **Timbre da instituição** que forneceu o comprovante;
+3. **Assinatura do responsável** pela instituição ou pela atividade;
+4. **Descrição das atividades** desenvolvidas pelo discente;
+5. **Data de início e término** da atividade;
+6. **Carga horária total** da atividade.</t>
+        </is>
+      </c>
+      <c r="K40" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L40" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2626,6 +3342,19 @@
         <v>0</v>
       </c>
       <c r="I41" t="b">
+        <v>1</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>De acordo com as normas do curso de Bacharelado em Estatística da UFBA, **não é permitido** em nenhuma das duas situações:
+1. **Acumular/computar uma mesma atividade em mais de uma modalidade:** Conforme estabelece expressamente o **Art. 6º da [Resolução Nº 03/2025, pág. 3](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)**, *"sob nenhuma hipótese serão computadas mais de uma vez atividades que pertençam a mais de uma das modalidades das AC definidas no Art. 3º desta resolução"*.
+2. **Usar horas de Atividades Complementares (AC) para dispensar disciplinas:** Conforme determina o **Art. 7º da [Resolução Nº 03/2025, pág. 3](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)**, *"atividades que foram aproveitadas como carga horária complementar não poderão ser utilizadas para dispensa de carga horária de outra natureza, como obrigatória, optativa e componente livre"*.</t>
+        </is>
+      </c>
+      <c r="K41" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L41" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2687,6 +3416,24 @@
       <c r="I42" t="b">
         <v>0</v>
       </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 3º da [Resolução nº 03/2025 do Colegiado do Curso de Bacharelado em Estatística](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)** (págs. 2 e 4-9), as experiências e vivências acadêmicas são reconhecidas em **seis modalidades** de Atividades Complementares. 
+Abaixo estão listadas as seis modalidades e os seus respectivos **limites máximos de carga horária** permitidos globalmente em cada uma delas, conforme estabelecido no Anexo 1 da referida resolução:
+1. **Ensino** — Carga horária máxima: **120 horas** (pág. 4)
+2. **Pesquisa** — Carga horária máxima: **120 horas** (pág. 4)
+3. **Extensão** — Carga horária máxima: **120 horas** (pág. 5)
+4. **Vivência Profissional** — Carga horária máxima: **90 horas** (pág. 8)
+5. **Programas Especiais** — Carga horária máxima: **120 horas** (pág. 8)
+6. **Representação Estudantil** — Carga horária máxima: **30 horas** (pág. 9)</t>
+        </is>
+      </c>
+      <c r="K42" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L42" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2746,6 +3493,28 @@
       <c r="I43" t="b">
         <v>0</v>
       </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da **Resolução nº 03/2025** do Colegiado do Curso de Bacharelado em Estatística da UFBA (que regulamenta as Atividades Complementares), o cálculo da carga horária e os tetos máximos para a modalidade **Ensino** são estabelecidos da seguinte forma para cada categoria:
+1. **Disciplinas cursadas com aprovação em outras instituições de ensino superior (que não fazem parte da grade curricular do Curso de Estatística):**
+   - **Cálculo da carga horária:** Aproveitamento integral da carga horária da disciplina cursada.
+   - **Teto máximo por atividade:** 90 horas.
+2. **Intercâmbio:**
+   - **Cálculo da carga horária:** Carga horária das disciplinas cursadas no intercâmbio (conforme documento emitido pela Instituição informando a carga horária total das disciplinas).
+   - **Teto máximo por atividade:** 90 horas.
+3. **PROFICI (Programa de Proficiência em Língua Estrangeira):**
+   - **Cálculo da carga horária:** Carga horária do curso por semestre.
+   - **Teto máximo por atividade:** 60 horas.
+*(Nota: O teto máximo global para a modalidade completa de **Ensino** é de **120 horas**).*
+Você pode consultar os detalhes na íntegra no documento oficial: [Resolução nº 03/2025 - Atividades Complementares (Anexo 1, págs. 4-6)](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf).</t>
+        </is>
+      </c>
+      <c r="K43" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="L43" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2801,6 +3570,26 @@
         <v>0</v>
       </c>
       <c r="I44" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da [Resolução nº 03/2025 do Colegiado do Curso de Bacharelado em Estatística da UFBA](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf) (págs. 4-8), a diferença no aproveitamento de horas para a **Modalidade Pesquisa** (que possui carga horária máxima de 120 horas) entre a participação em projeto de pesquisa comum e a realização de Iniciação Científica ou programas institucionais ocorre nos seguintes pontos:
+1. **Participação em Projeto de Pesquisa coordenado por docente da UFBA** (diferente de Iniciação Científica e/ou similares):
+   * **Carga horária concedida:** 15 horas por semestre (ou o equivalente a 1/6 das 15 horas por mês).
+   * **Carga horária máxima para a atividade:** 30 horas.
+   * **Requisito/Documentação:** Declaração emitida pelo docente coordenador registrando carga horária mínima de 20 horas por semestre (Conforme o Anexo 1, pág. 4).
+2. **Realização de trabalho de pesquisa ou Iniciação Científica (IC) ou Permanecer (Linha Pesquisa) ou SANKOFA (Linha Pesquisa)**, sob orientação de docente da UFBA:
+   * **Carga horária concedida:** 45 horas por semestre.
+   * **Carga horária máxima para a atividade:** 90 horas.
+   * **Requisito/Documentação:** Certificado ou declaração da atividade explicitando o título do trabalho, a carga horária total e o período de realização (Conforme o Anexo 1, pág. 4).
+*(Nota: Caso os programas Permanecer e SANKOFA sejam realizados na Linha Extensão, eles possuem regras e limites próprios previstos na modalidade Extensão, pontuando 60 horas por semestre até o máximo de 120 horas, conforme consta na página 7 do mesmo anexo).*</t>
+        </is>
+      </c>
+      <c r="K44" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="L44" t="b">
         <v>0</v>
       </c>
     </row>
@@ -2860,6 +3649,27 @@
         <v>0</v>
       </c>
       <c r="I45" t="b">
+        <v>1</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da **Resolução nº 03/2025** do Colegiado do Curso de Bacharelado em Estatística da UFBA, que regulamenta as Atividades Complementares (págs. 4-5), as cargas horárias atribuídas na modalidade **Pesquisa** são as seguintes:
+1. **Trabalho publicado em periódico que possua corpo editorial:**
+   - **Carga horária por atividade:** 45 horas por trabalho.
+   - **Carga horária máxima para a atividade:** 90 horas.
+2. **Apresentação de trabalhos (oral ou pôster) em eventos científicos:**
+   - **Carga horária por atividade:** 10 horas por trabalho.
+   - **Carga horária máxima para a atividade:** 40 horas.
+3. **Participação em eventos científicos como ouvinte (congressos, seminários, oficinas, encontros e similares):**
+   - **Carga horária por atividade:** Até 5 horas por dia por evento.
+   - **Carga horária máxima para a atividade:** 80 horas.
+Você pode consultar o teor completo e as regras de comprovação no documento oficial: [Resolução nº 03/2025 - Atividades Complementares (págs. 4-5)](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf).</t>
+        </is>
+      </c>
+      <c r="K45" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L45" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2927,6 +3737,40 @@
       <c r="I46" t="b">
         <v>0</v>
       </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da **Resolução nº 03/2025** do Colegiado do Curso de Bacharelado em Estatística da UFBA, os limites por semestre e os limites totais de carga horária para Atividades Complementares (AC) diferem entre a atuação em Empresa Júnior (classificada na modalidade **Extensão**) e as atividades da modalidade **Vivência Profissional**:
+### 1. Prestação de Serviços em Empresa Júnior (Modalidade Extensão)
+* **Limite por semestre:** Máximo de **30 horas por semestre**.
+* **Limite total (máximo aproveitado para a atividade):** Até **120 horas** (dentro do teto geral da modalidade de Extensão, que possui carga horária máxima de 120 horas).
+* **Documentação exigida:** Certificado ou declaração assinada pelo professor tutor, explicitando as atividades desenvolvidas, a carga horária e o período de realização da atividade ([Resolução nº 03/2025, Anexo 1, pág. 5](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).
+---
+### 2. Atuação na Modalidade Vivência Profissional
+A modalidade de **Vivência Profissional** possui uma carga horária máxima total de **90 horas** ([Resolução nº 03/2025, Anexo 1, pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)). Ela contempla diferentes tipos de atuação com limites específicos por atividade:
+* **Atividades em empresas juniores na UFBA:** 
+  * *Limite por semestre:* Máximo de **20 horas por semestre** (com exigência de relatório do professor responsável atestando carga horária mínima de 45 horas de trabalhos realizados no período).
+  * *Limite total:* Até **60 horas**.
+  * *Documentação exigida:* Relatório do professor responsável pela Empresa Júnior avaliando a atuação e o aproveitamento do discente ([Resolução nº 03/2025, Anexo 1, pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).
+* **Estágio não-obrigatório** (que respeite as Normas de Estágio do IME):
+  * *Limite por semestre:* **30 horas por semestre**.
+  * *Limite total:* Até **90 horas**.
+  * *Documentação exigida:* Termo de compromisso e relatório de conclusão da atividade com assinatura dos responsáveis ([Resolução nº 03/2025, Anexo 1, pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).
+* **Trabalho relacionado com Estatística:**
+  * *Limite por semestre:* **25 horas por semestre**.
+  * *Limite total:* Até **75 horas**.
+  * *Documentação exigida:* Declaração emitida e assinada pelo superior imediato informando as atividades desenvolvidas ([Resolução nº 03/2025, Anexo 1, pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).
+* **Trabalho não relacionado com Estatística:**
+  * *Limite por semestre:* **15 horas por semestre**.
+  * *Limite total:* Até **60 horas**.
+  * *Documentação exigida:* Declaração emitida e assinada pelo superior imediato informando as atividades desenvolvidas ([Resolução nº 03/2025, Anexo 1, pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="L46" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2981,6 +3825,23 @@
         <v>0</v>
       </c>
       <c r="I47" t="b">
+        <v>1</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da **Resolução nº 03/2025** do Colegiado do Curso de Bacharelado em Estatística da UFBA ([Resolução_03_2025_Atividades_Complementares_SIGAA, págs. 5-6](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)), as cargas horárias atribuídas por semestre e os limites máximos para essas atividades extensionistas são os seguintes:
+1. **Atuação em atividades de extensão desenvolvidas em centros de estudos e laboratórios vinculados ao Instituto de Matemática e Estatística (IME) da UFBA ou a outras unidades da UFBA, cadastrados no SIATEX:**
+   - **Carga horária por semestre:** Máximo de **45 horas por semestre**.
+   - **Carga horária máxima aproveitada na modalidade:** **90 horas**.
+2. **Atuação como Monitor em ACCS (Ação Curricular em Comunidade e Sociedade):**
+   - **Carga horária por semestre:** **60 horas por semestre**.
+   - **Carga horária máxima aproveitada na modalidade:** **90 horas**.</t>
+        </is>
+      </c>
+      <c r="K47" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L47" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3050,6 +3911,32 @@
         <v>1</v>
       </c>
       <c r="I48" t="b">
+        <v>1</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da [Resolução Nº 03/2025 do Colegiado do Curso de Bacharelado em Estatística da UFBA (págs. 7-9)](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf), as cargas horárias computadas na modalidade **Extensão** para as referidas atividades são:
+*   **Bolsistas PIBIEX:** 
+    *   **Por semestre:** 60 horas por semestre.
+    *   **Total máximo:** 120 horas.
+*   **Bolsista de Projeto do PAEX:** 
+    *   **Por semestre:** 60 horas por semestre.
+    *   **Total máximo:** 120 horas.
+*   **Permanecer (Linha Extensão):** 
+    *   **Por semestre:** 60 horas por semestre.
+    *   **Total máximo:** 120 horas.
+*   **SANKOFA (Linha Extensão):** 
+    *   **Por semestre:** 60 horas por semestre.
+    *   **Total máximo:** 120 horas.
+*   **Liga Acadêmica:** 
+    *   **Por semestre:** 30 horas por semestre.
+    *   **Total máximo:** 90 horas.</t>
+        </is>
+      </c>
+      <c r="K48" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L48" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3124,6 +4011,37 @@
       <c r="I49" t="b">
         <v>0</v>
       </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Com base no **Anexo 1** da [Resolução nº 03/2025 do Colegiado do Curso de Bacharelado em Estatística da UFBA](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf) (págs. 7-8), que regulamenta as Atividades Complementares (AC) na modalidade **Vivência Profissional** (cuja carga horária total máxima acumulada na modalidade é de **90 horas**), as exigências de cargas horárias, limites e documentações para cada uma das categorias são as seguintes:
+---
+### 1. Estágio não obrigatório
+* **Carga horária semestral:** 30 horas por semestre.
+* **Limite máximo (por atividade):** 90 horas.
+* **Documentos exigidos:** 
+  * Termo de Compromisso de Estágio;
+  * Relatório de conclusão da atividade com assinatura dos responsáveis pela atividade.
+  *(Conforme previsto também nas [Resoluções nº 01 e 02/2020 de Estágio Não Obrigatório do IME](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)), o estágio deve respeitar as Normas de Estágio do IME ou do Colegiado de Estatística, exigindo prévio convênio, plano de estágio e relatórios periódicos.*
+### 2. Trabalho relacionado com Estatística
+* **Carga horária semestral:** 25 horas por semestre.
+* **Limite máximo (por atividade):** 75 horas.
+* **Documentos exigidos:** 
+  * Declaração emitida e assinada pelo superior imediato, informando as atividades desenvolvidas pelo funcionário.
+### 3. Trabalho não relacionado com Estatística
+* **Carga horária semestral:** 15 horas por semestre.
+* **Limite máximo (por atividade):** 60 horas.
+* **Documentos exigidos:** 
+  * Declaração emitida e assinada pelo superior imediato, informando as atividades desenvolvidas pelo funcionário.
+---
+*(Nota complementar extraída do mesmo Anexo 1, pág. 8: Caso a atividade envolva **Empresas Juniores na UFBA**, a carga horária considerada é de 20 horas por semestre, com limite máximo de 60 horas, exigindo relatório do professor responsável pela Empresa Júnior avaliando a atuação do discente com aproveitamento e carga horária mínima de 45 horas por semestre de trabalhos realizados).*</t>
+        </is>
+      </c>
+      <c r="K49" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L49" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3180,6 +4098,28 @@
       <c r="I50" t="b">
         <v>0</v>
       </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da [Resolução nº 03/2025 do Colegiado do Curso de Bacharelado em Estatística da UFBA](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf) (págs. 7-9), a contabilização e as regras para a modalidade **Programas Especiais** (que possui carga horária máxima permitida de **120 horas** para a modalidade) ocorrem da seguinte forma:
+1. **Programa Especial de Treinamento (PET)**:
+   - **Contabilização:** Carga horária total de **30 horas por semestre de atividade**, ou o equivalente a **1/6 das 30 horas por mês**.
+   - **Carga horária máxima aproveitada para a atividade:** **60 horas** ([págs. 7 e 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).
+   - **Comprovação:** Certificado ou declaração da atividade explicitando o título do trabalho, a carga horária total e o período de realização.
+2. **Monitoria**:
+   - **Contabilização:** Carga horária total de **30 horas por semestre de atividade**, ou o equivalente a **1/6 das 30 horas por mês** (conforme tabela da pág. 8).
+   - **Carga horária máxima aproveitada para a atividade:** **60 horas** ([pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).
+   - **Comprovação:** Certificado ou declaração da atividade explicitando o título do trabalho, a carga horária total e o período de realização.
+3. **Outros Programas Especiais (Permanecer, SANKOFA em linhas de Ensino/Pesquisa ou Participação em Programas Especiais oferecidos pela UFBA)**:
+   - **Permanecer / SANKOFA (Linha Ensino ou Pesquisa):** Contabilizados em **45 horas por semestre**, com limite máximo de **90 horas** para a atividade ([pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).
+   - **Participação em Programas Especiais oferecidos pela UFBA** (não contemplados na modalidade de Extensão e não mencionados acima): Carga horária total de **30 horas por semestre de atividade** (ou o equivalente a 1/6 das 30 horas por mês), com limite máximo de **60 horas** ([pág. 9](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf)).</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L50" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3233,6 +4173,24 @@
         <v>0</v>
       </c>
       <c r="I51" t="b">
+        <v>0</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Com base na **Resolução nº 03/2025** do Colegiado do Curso de Bacharelado em Estatística da UFBA, que regulamenta as Atividades Complementares (AC), as regras referentes à representação discente (incluindo carga horária por mandato, limites e documentação) são as seguintes:
+1. **Representação discente em órgãos colegiados no âmbito da UFBA:**
+   - **Carga horária concedida:** 15 horas por mandato (com limite máximo total da modalidade "Representação Estudantil" fixado em 30 horas, conforme a pág. 9 do Anexo 1).
+   - **Documentação exigida:** Declaração do órgão colegiado.
+2. **Representação discente na UFBA (CA, DA e/ou DCE):**
+   - **Carga horária concedida:** 15 horas por mandato (com limite máximo total da modalidade "Representação Estudantil" fixado em 30 horas, conforme a pág. 9 do Anexo 1).
+   - **Documentação exigida:** Ata de posse e declaração do órgão discente de cumprimento da representação.
+Para mais detalhes, consulte o documento oficial na íntegra: [Resolução nº 03/2025 - Atividades Complementares do Curso de Estatística da UFBA, págs. 7-9](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf).</t>
+        </is>
+      </c>
+      <c r="K51" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L51" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3306,6 +4264,35 @@
       <c r="I52" t="b">
         <v>0</v>
       </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo 1** da [Resolução nº 03/2025 do Colegiado do Curso de Bacharelado em Estatística da UFBA (pág. 9)](https://colest.ime.ufba.br/wp-content/uploads/2026/10/Resolucao_03_2025_Atividades_Complementares_SIGAA_assinado.pdf), a modalidade **Representação Estudantil** possui uma **carga horária máxima total de 30 horas** que podem ser aproveitadas na integralização. 
+A distribuição de horas e os limites específicos para as diferentes funções de participação na Atlética IME dentro desta modalidade ocorrem da seguinte forma:
+1. **Participação Atlética IME - Diretoria (Presidente, Vice-Presidente e Diretorias):**
+   * **Distribuição:** 20 horas por semestre.
+   * **Limite máximo:** 40 horas.
+   * **Documentação exigida:** Certificado ou declaração de participação com registro de data e carga horária.
+2. **Participação Atlética IME - Assistência de Diretoria:**
+   * **Distribuição:** 10 horas por semestre.
+   * **Limite máximo:** 20 horas.
+   * **Documentação exigida:** Certificado ou declaração de participação com registro de data e carga horária.
+3. **Participação Atlética IME - Representantes de modalidades esportivas:**
+   * **Distribuição:** 4 horas por semestre.
+   * **Limite máximo:** 8 horas.
+   * **Documentação exigida:** Certificado ou declaração de participação com registro de data e carga horária.
+4. **Participação Atlética IME - Atleta:**
+   * **Distribuição:** 5 horas por campeonato/torneio.
+   * **Limite máximo:** 20 horas.
+   * **Documentação exigida:** Certificado ou declaração de participação com registro de data e carga horária.
+Vale ressaltar que, conforme o **Parágrafo único do Art. 1º** e o **§ 2º do Art. 5º** da mesma resolução, a pontuação a ser adicionada no sistema acadêmico respeitará o limite máximo estabelecido para a modalidade e para cada atividade específica.</t>
+        </is>
+      </c>
+      <c r="K52" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="L52" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3351,6 +4338,20 @@
       <c r="I53" t="b">
         <v>0</v>
       </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>De acordo com a regulamentação específica do Bacharelado em Estatística da UFBA:
+* **Códigos das disciplinas obrigatórias do TCC:** O Trabalho de Conclusão de Curso é desenvolvido nas disciplinas obrigatórias **MATD52** (Trabalho de Conclusão de Curso I - TCCI) e **MATD53** (Trabalho de Conclusão de Curso II - TCCII).
+* **Resolução revogada:** A norma que normatiza estas atividades revogou explicitamente a **Resolução nº 04/2023**.
+Para mais detalhes, consulte a [Resolução nº 05/2024, págs. 1-2](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K53" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L53" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3395,6 +4396,20 @@
       </c>
       <c r="I54" t="b">
         <v>0</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>De acordo com a regulamentação do curso de Bacharelado em Estatística da UFBA, o Trabalho de Conclusão de Curso (TCC) pode ser apresentado e redigido nos seguintes formatos e idiomas:
+* **Formatos aceitos:** O TCC pode ser apresentado na forma de **trabalho monográfico** ou de **artigo científico**.
+* **Idiomas permitidos:** O texto do trabalho poderá ser redigido e apresentado tanto em **português** quanto em **inglês**.
+Essas diretrizes estão estabelecidas no **Art. 1º** e no **Art. 8º (Inciso I)** da [Resolução nº 05/2024, págs. 1 e 5](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K54" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L54" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="55">
@@ -3447,6 +4462,22 @@
       <c r="I55" t="b">
         <v>0</v>
       </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 2º da Resolução nº 05/2024** ([Resolução_05_2024_TCC_Estatistica, págs. 1-2](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)), são cinco as competências atribuídas ao Colegiado do Curso de Bacharelado em Estatística em relação à gestão do Trabalho de Conclusão de Curso (TCC):
+1. **Tornar públicas as normas do TCC** (Inciso I);
+2. **Divulgar, junto aos alunos, a relação dos professores orientadores e suas respectivas propostas de projetos** no semestre que antecede à matrícula na disciplina MATD52 (Inciso II);
+3. **Divulgar entre discentes do curso a apresentação de trabalho monográfico** das disciplinas MATD52 e MATD53 (Inciso III);
+4. **Arquivar a(s) ata(s) assinada(s) pela banca examinadora** (Anexo VI) **e cópia(s) digital do(s) trabalho(s) monográfico(s)** (Inciso IV);
+5. **Informar ao(à) professor(a) orientador(a) que a versão final do TCCII foi entregue ao Colegiado** (Inciso V).</t>
+        </is>
+      </c>
+      <c r="K55" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L55" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3489,6 +4520,21 @@
         <v>0</v>
       </c>
       <c r="I56" t="b">
+        <v>0</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>De acordo com a regulamentação do curso de Bacharelado em Estatística da UFBA, o estudante deve realizar os seguintes procedimentos no semestre anterior antes de se matricular na disciplina **MATD52 (Trabalho de Conclusão de Curso I - TCCI)**:
+1. **Contato prévio com um orientador:** O aluno deve contatar, com antecedência, um(a) professor(a) do Departamento de Estatística para atuar como possível orientador(a) da monografia ou artigo científico (*§ 1º do Art. 3º*).
+2. **Entrega do Termo de Aceite:** O discente deve entregar ao Colegiado de Estatística o **termo de aceite de orientação (Anexo I)** devidamente assinado pelo professor orientador, manifestando concordância com a orientação. Esse procedimento deve ser feito na data estipulada pelo coordenador, com base na agenda acadêmica (*§ 2º do Art. 3º*).
+3. **Divulgação prévia pelo Colegiado:** O Colegiado do curso é responsável por divulgar antecipadamente aos alunos a relação dos professores orientadores e suas respectivas propostas de projetos no semestre que antecede a matrícula (*Inciso II do Art. 2º*).
+Todas essas diretrizes constam na [Resolução nº 05/2024, págs. 1-2](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K56" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="L56" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3539,6 +4585,24 @@
         <v>0</v>
       </c>
       <c r="I57" t="b">
+        <v>0</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>De acordo com a [Resolução nº 05/2024 do Colegiado do Curso de Bacharelado em Estatística da UFBA](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), os procedimentos para cursar a disciplina **MATD53 (Trabalho de Conclusão de Curso II)** no semestre seguinte e as regras em caso de mudança de orientador são os seguintes:
+### 1. Como proceder para cursar a disciplina MATD53 no semestre seguinte:
+* **Manifestação de interesse:** De acordo com o **§ 3º do Art. 3º** da resolução (págs. 2-3), os alunos que cursarão a disciplina MATD53 no semestre subsequente deverão manifestar o seu interesse no período de pré-matrícula, junto ao seu orientador acadêmico.
+* **Renovação:** O orientador deverá assinar o termo correspondente (**Termo de Renovação de TCC II - Anexo II**, pág. 8) no semestre que antecede a disciplina MATD53, conforme o **Inciso II do Art. 5º** (pág. 2).
+### 2. O que é exigido caso ocorra mudança de orientador entre as disciplinas:
+* **Regra geral e exceções:** O **§ 4º do Art. 3º** (pág. 2) estabelece que o professor orientador da disciplina MATD52 (TCC I) deverá ser o mesmo na disciplina MATD53 (TCC II), salvo em **casos excepcionais** devidamente informados ao Colegiado.
+* **Formalização da mudança:** Conforme o **§ 5º do Art. 3º** e o **Inciso III do Art. 5º** (págs. 2 e 5), no caso de mudança de orientação e/ou coorientação, o aluno e o novo orientador deverão formalizar a alteração entregando ao Colegiado de Estatística o **Termo de Aceite de Orientação de TCC II (Anexo III)** devidamente assinado no semestre que antecede a disciplina MATD53.
+Para mais detalhes e acesso aos modelos dos anexos, consulte a [Resolução nº 05/2024, págs. 1-8](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K57" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="L57" t="b">
         <v>0</v>
       </c>
     </row>
@@ -3591,6 +4655,19 @@
       <c r="I58" t="b">
         <v>0</v>
       </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>De acordo com a [Resolução nº 05/2024 (pág. 2)](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), que normatiza as atividades de TCC do curso de Bacharelado em Estatística da UFBA:
+* **Orientador(a):** Deve ser obrigatoriamente **professor(a) do Departamento de Estatística** da universidade (conforme o Art. 4º da [Resolução nº 05/2024, pág. 2](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)).
+* **Coorientador(a):** A coorientação é permitida a **professores de instituições de ensino superior** e, em **casos especiais, a profissionais com nível superior** de instituições de reconhecida competência na área de estudo do TCC. Para isso, é necessária a entrega do termo de aceite assinado pelo orientador (Anexo I ou Anexo II), conforme o parágrafo único do Art. 4º da [Resolução nº 05/2024 (pág. 2)](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K58" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L58" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3640,6 +4717,21 @@
       <c r="I59" t="b">
         <v>0</v>
       </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>De acordo com a **Resolução nº 05/2024** do Colegiado do Curso de Bacharelado em Estatística da UFBA, que normatiza as atividades de TCC (MATD52 e MATD53), os termos formais que o professor orientador deve assinar no semestre que antecede cada disciplina são:
+1. **No semestre que antecede a disciplina MATD52 (TCC I):** O professor orientador deve assinar o **Termo de Aceite** (conforme o **Anexo I** da resolução), manifestando sua concordância com a orientação do discente (Art. 3º, § 2º e Art. 5º, inciso I, págs. 1-2).
+2. **No semestre que antecede a disciplina MATD53 (TCC II):** O professor orientador deve assinar o **Termo de Renovação** (conforme o **Anexo II** da resolução), ou o **Termo de Aceite** (conforme o **Anexo III**) caso ocorra mudança de orientação e/ou coorientação (Art. 5º, inciso II e Art. 5º, inciso III do Capítulo II, págs. 2-3).
+Você pode consultar o documento completo e seus respectivos anexos diretamente no link oficial:
+[Resolução nº 05/2024 - Normas de TCC do Bacharelado em Estatística da UFBA, págs. 1-8](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K59" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L59" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3684,6 +4776,19 @@
       <c r="I60" t="b">
         <v>0</v>
       </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>De acordo com a [Resolução nº 05/2024 do Colegiado do Curso de Bacharelado em Estatística](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), as antecedências mínimas que o professor orientador deve observar são as seguintes:
+1. **Membros da banca examinadora:** O orientador deve informar ao Colegiado do Curso, com antecedência mínima de **20 dias**, os nomes de quatro possíveis membros da banca examinadora que participarão da avaliação das disciplinas MATD52 (TCCI) e MATD53 (TCCII), conforme o inciso VI do Art. 5º (pág. 3) e o Anexo IV (pág. 8).
+2. **Data, hora e local da defesa:** O orientador deve informar ao Colegiado, com antecedência mínima de **15 dias**, sobre a data, a hora e o local da defesa do projeto ou trabalho final de TCC, conforme o inciso VII do Art. 5º (pág. 3).</t>
+        </is>
+      </c>
+      <c r="K60" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L60" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3727,6 +4832,18 @@
       <c r="I61" t="b">
         <v>1</v>
       </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>De acordo com o **Inciso VIII do Artigo 5º** da [Resolução nº 05/2024 (págs. 1 e 3)](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf) do Colegiado do Curso de Bacharelado em Estatística da UFBA, é competência do professor orientador:
+&gt; "providenciar a entrega das cópias do projeto e/ou do trabalho monográfico à banca examinadora, no **mínimo quinze dias antes** da data do ato público;"</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L61" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3765,6 +4882,19 @@
         <v>1</v>
       </c>
       <c r="I62" t="b">
+        <v>1</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>De acordo com a [Resolução nº 05/2024 do Colegiado do Curso de Estatística](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), o(a) professor(a) orientador(a) está autorizado(a) a registrar a nota final da disciplina **MATD53** (Trabalho de Conclusão de Curso II - TCCII) no Sistema Acadêmico **após a informação do Colegiado de que o aluno entregou a versão final do trabalho monográfico**.
+Conforme detalhado no documento:
+- **Origem e dispositivo:** Inciso XII do Art. 5º da [Resolução nº 05/2024, página 3 (fichamento e texto regulamentar)](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K62" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L62" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3809,6 +4939,18 @@
         <v>1</v>
       </c>
       <c r="I63" t="b">
+        <v>1</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>De acordo com o **Inciso II do Artigo 6º** do Capítulo III da **Resolução nº 05/2024** do Colegiado do Curso de Bacharelado em Estatística da UFBA, compete ao aluno enviar o projeto ou o trabalho monográfico ao orientador com a antecedência mínima de **20 (vinte) dias** antes da data do ato público para as apresentações.
+Além disso, cabe destacar que o **Inciso VIII do Artigo 5º** estabelece que é responsabilidade do professor orientador providenciar a entrega das cópias do projeto ou do trabalho monográfico à banca examinadora no mínimo **15 (quinze) dias** antes da data do ato público (págs. 1-3 da [Resolução nº 05/2024, págs. 1-3](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)).</t>
+        </is>
+      </c>
+      <c r="K63" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L63" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3859,6 +5001,19 @@
       <c r="I64" t="b">
         <v>0</v>
       </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>De acordo com o **Inciso IV do Art. 6º da [Resolução nº 05/2024 do Colegiado do Curso de Estatística da UFBA](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)** (página 2 do documento), o prazo máximo e o formato exigidos são os seguintes:
+* **Prazo máximo:** No máximo **quinze dias** após a defesa.
+* **Formato exigido:** Uma cópia digital (em formato PDF) da versão final do trabalho monográfico, que deve ser entregue no Colegiado do Curso acompanhada pela respectiva autorização ([Anexo IV](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)).</t>
+        </is>
+      </c>
+      <c r="K64" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L64" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3899,6 +5054,17 @@
       </c>
       <c r="I65" t="b">
         <v>0</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>De acordo com o **§ 1º do Art. 6º da Resolução nº 05/2024** do Colegiado do Curso de Bacharelado em Estatística da UFBA ([Resolução nº 05/2024, pág. 2](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)), o estudante que não comparecer ao ato público para a defesa do seu projeto ou trabalho monográfico será **reprovado na disciplina** (MATD52 ou MATD53), **salvo** se apresentar uma justificativa prevista no **Art. 115 do Regulamento de Ensino de Graduação e Pós-Graduação (REGPG)** da UFBA.</t>
+        </is>
+      </c>
+      <c r="K65" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L65" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
@@ -3950,6 +5116,20 @@
       <c r="I66" t="b">
         <v>0</v>
       </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 7º da [Resolução nº 05/2024](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)** (págs. 2-3 do documento / pág. 2 da visualização), a banca examinadora do TCCI e do TCCII deve ser composta por **três membros**, indicados pelo professor orientador. 
+No que tange à exigência de vínculo com o Departamento de Estatística, o parágrafo único do mesmo artigo estabelece os seguintes critérios:
+* No mínimo **dois professores devem ser membros do Departamento de Estatística da UFBA**, o que já inclui o próprio orientador.
+* Caso haja orientador e coorientador, **apenas um deles poderá compor a banca** examinadora.</t>
+        </is>
+      </c>
+      <c r="K66" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L66" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3991,6 +5171,18 @@
       </c>
       <c r="I67" t="b">
         <v>1</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>De acordo com o **Parágrafo único, inciso II do Art. 7º da Resolução nº 05/2024**, que normatiza as atividades de Trabalho de Conclusão de Curso (TCC) do Bacharelado em Estatística da UFBA, **não é permitido**. O regulamentou estabelece expressamente que, na existência de orientador e coorientador, **apenas um deles poderá compor a banca**.
+Você pode conferir essa diretriz diretamente no documento oficial: [Resolução nº 05/2024 do Colegiado do Curso de Estatística, pág. 2](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).</t>
+        </is>
+      </c>
+      <c r="K67" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L67" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="68">
@@ -4041,6 +5233,22 @@
       <c r="I68" t="b">
         <v>0</v>
       </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>De acordo com o **Artigo 8º do Capítulo V** da [Resolução nº 05/2024](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), o Trabalho de Conclusão de Curso (TCC) deve apresentar as seguintes exigências quanto ao conteúdo e às características textuais e bibliográficas (pág. 2):
+I. Ser redigido e apresentado em **português ou em inglês**;
+II. O texto deverá ser **original**, relacionado com a investigação científica teórica ou aplicada, na área de Estatística;
+III. Ter caráter eminentemente **acadêmico**, visando à investigação científica;
+IV. Ser fruto de **reflexão e rigor científico**, não devendo constituir-se em mero acervo de transcrições de trabalhos alheios;
+V. Possuir **formatação e referências bibliográficas segundo as normas da ABNT**.</t>
+        </is>
+      </c>
+      <c r="K68" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="L68" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4085,6 +5293,19 @@
       <c r="I69" t="b">
         <v>1</v>
       </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 9º** da [Resolução nº 05/2024 do Colegiado do Curso de Estatística, págs. 2-3](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), o tempo regulamentar de apresentação oral do estudante nas defesas das disciplinas de Trabalho de Conclusão de Curso é o seguinte:
+* **Disciplina MATD52 (Trabalho de Conclusão de Curso I - TCCI):** O tempo de apresentação do projeto de trabalho monográfico será de **15 a 20 minutos** (§ 1º do Art. 9º).
+* **Disciplina MATD53 (Trabalho de Conclusão de Curso II - TCCII):** O tempo de apresentação do trabalho monográfico será de **25 a 30 minutos** (§ 2º do Art. 9º).</t>
+        </is>
+      </c>
+      <c r="K69" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L69" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4128,6 +5349,19 @@
       <c r="I70" t="b">
         <v>0</v>
       </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>De acordo com a regulamentação específica do Trabalho de Conclusão de Curso do Bacharelado em Estatística da UFBA, o cálculo da nota final e os critérios de aprovação para as disciplinas **MATD52** (Trabalho de Conclusão de Curso I - TCCI) e **MATD53** (Trabalho de Conclusão de Curso II - TCCII) seguem o estabelecido no **§ 3º do Art. 9º da [Resolução nº 05/2024, página 3](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)**:
+* **Cálculo da Nota Final:** A nota final do discente em ambas as disciplinas é calculada por meio da **média aritmética simples** das notas atribuídas pelos membros da banca examinadora.
+* **Média Mínima para Aprovação:** O(a) aluno(a) será considerado(a) **aprovado(a)** quando a média de suas notas for **maior ou igual a 5,0 (cinco)**.</t>
+        </is>
+      </c>
+      <c r="K70" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L70" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4169,6 +5403,19 @@
         <v>1</v>
       </c>
       <c r="I71" t="b">
+        <v>0</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 10 da [Resolução nº 05/2024 (Normas de TCC do Bacharelado em Estatística da UFBA), pág. 3](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf)**, caso seja comprovada a existência de fraude ou plágio (parcial ou total), as seguintes consequências são previstas:
+* O trabalho será **reprovado por infração à ética acadêmica** (Capítulo VI, Art. 10).
+* Além disso, conforme o **parágrafo único** do mesmo artigo, o Colegiado poderá instaurar uma **comissão de sindicância**, de acordo com as leis específicas aplicáveis.</t>
+        </is>
+      </c>
+      <c r="K71" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L71" t="b">
         <v>0</v>
       </c>
     </row>
@@ -4237,6 +5484,34 @@
       <c r="I72" t="b">
         <v>0</v>
       </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo IV (Parecer de Autorização para Apresentação do TCCI/TCCII)** da [Resolução nº 05/2024 do Colegiado do Curso de Bacharelado em Estatística da UFBA (págs. 9, 12)](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), o formulário é composto pelas seguintes informações e sugestões de nomes:
+### **Informações que compõem o formulário:**
+1. **Identificação do(a) Orientador(a) e do(a) Discente:** Nome do(a) professor(a) orientador(a), nome completo do(a) discente, número de matrícula e indicação se a autorização refere-se à disciplina de TCC I ou TCC II (`I/II`).
+2. **Título do Trabalho:** O título do projeto ou trabalho monográfico.
+3. **Natureza do Trabalho:** Indicação se o documento avaliado constitui um "projeto" ou um "trabalho".
+4. **Logística da Apresentação:**
+   * **Data prevista** da apresentação.
+   * **Horário previsto** da apresentação (intervalo de início e término, em horas).
+   * **Local previsto** (dados da sala física ou virtual).
+5. **Local, Data e Assinatura:** Cidade (Salvador), dia, mês, ano e a assinatura com o nome do(a) professor(a) orientador(a).
+---
+### **Quantas e quais sugestões de nomes compõem a banca:**
+O formulário prevê o preenchimento de **5 (cinco) sugestões de nomes** para compor a banca examinadora, detalhadas da seguinte forma:
+* **a)** 1 (um) nome para **Orientador(a) / Coorientador(a)**;
+* **b)** 1 (um) nome de membro **titular** (com a respectiva identificação da lotação);
+* **c)** 1 (um) nome de membro **titular** (com a respectiva identificação da lotação);
+* **d)** 1 (um) nome de membro **suplente** (com a respectiva identificação da lotação);
+* **e)** 1 (um) nome de membro **suplente** (com a respectiva identificação da lotação).</t>
+        </is>
+      </c>
+      <c r="K72" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="L72" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4285,6 +5560,20 @@
       <c r="I73" t="b">
         <v>0</v>
       </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>De acordo com o **Anexo VII** da [Resolução nº 05/2024 (págs. 4-4)](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), o **Termo de Autorização para Publicação do TCC** estabelece que o(a) discente, na qualidade de titular dos direitos de autor da publicação, autoriza o Colegiado do Curso de Bacharelado em Estatística da UFBA a disponibilizar o texto integral de sua obra (trabalho monográfico ou artigo científico) no sítio eletrônico do colegiado (`https://colest.ime.ufba.br/`). Essa publicação ocorre sem o pagamento de quaisquer direitos autorais patrimoniais, em conformidade com a Lei nº 9.610/98, com o objetivo de divulgar a produção científica dos(as) alunos(as) do curso. O documento também permite definir a data a partir da qual o trabalho poderá ser disponibilizado no website.
+O referido documento exige as seguintes assinaturas:
+1. **Assinatura do(a) autor(a)** (o(a) discente), acompanhada do nome completo, local e data.
+2. **Assinatura do(a) orientador(a)** (anuência), acompanhada do nome completo, local e data.</t>
+        </is>
+      </c>
+      <c r="K73" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L73" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -4331,6 +5620,18 @@
       <c r="I74" t="b">
         <v>0</v>
       </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>De acordo com a [Resolução nº 05/2024 do Colegiado do Curso de Estatística](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf), o documento apresentado no **Anexo V** (pág. 12 do documento oficial / pág. 2 da visualização) corresponde ao **"Parecer de Autorização para Entrega do TCCII"**. 
+Sua finalidade é formalizar a autorização por parte do(a) professor(a) orientador(a) para que o(a) aluno(a) realize a entrega da versão final do seu trabalho monográfico (TCCII) ao Colegiado do Curso de Estatística.</t>
+        </is>
+      </c>
+      <c r="K74" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L74" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4374,6 +5675,22 @@
       <c r="I75" t="b">
         <v>0</v>
       </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>De acordo com os documentos normativos do curso de Estatística da UFBA, há menções a diferentes resoluções com Anexos III. Abaixo estão os documentos correspondentes encontrados:
+1. **Resolução de TCC (Resolução nº 05/2024)**: O documento constante no **Anexo III** formaliza o **Termo de Aceite de Orientação de TCC II** (referente à disciplina MATD52/MATD53 – Trabalho de Conclusão de Curso II). Por meio deste termo, o(a) professor(a) orientador(a) do Instituto de Matemática e Estatística da UFBA declara formalmente que aceita orientar o(a) discente na elaboração do TCC II, especificando o semestre de início, eventuais coorientadores e a ciência das normas que regulamentam a atividade no Curso de Estatística.
+   - Fonte: [Resolução_05_2024_TCC_Estatistica, pág. 8](https://colest.ime.ufba.br/wp-content/uploads/2025/01/Resolucao_05_2024_TCC.pdf).
+2. **Resoluções de Estágio Não Obrigatório do IME (Resoluções nº 01 e 02/2020)**: Caso você esteja se referindo às normas complementares de estágio e seus anexos correlatos de formulários e controle (como o Anexo A de Plano de Estágio, Anexo B de Relatório e Anexo C de Rescisão), estes formalizam, respectivamente, o planejamento das atividades supervisionadas, a avaliação periódica do estagiário e a rescisão formal do Termo de Compromisso de Estágio com a interveniência da UFBA.
+   - Fonte: [Resolucoes_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 7-13](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf).
+Caso precise de detalhes sobre um anexo específico de outra resolução não listada acima, por favor, informe o nome exato da norma para nova verificação.</t>
+        </is>
+      </c>
+      <c r="K75" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="L75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4417,6 +5734,18 @@
       <c r="I76" t="b">
         <v>1</v>
       </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>De acordo com o **Inciso II do Art. 2º da Resolução nº 01/2020** do Instituto de Matemática e Estatística da UFBA, o Termo de Compromisso deve ser emitido em **pelo menos 3 vias**, devendo estar assinado pelo representante legal da instituição cedente (com carimbo), pelo estudante e, de forma opcional, por duas testemunhas.
+Você pode consultar os detalhes na íntegra no documento [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME (pág. 2)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf).</t>
+        </is>
+      </c>
+      <c r="K76" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L76" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4458,6 +5787,19 @@
         <v>1</v>
       </c>
       <c r="I77" t="b">
+        <v>1</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>De acordo com o **Parágrafo único do Art. 14º** do Capítulo VII da [Resolução Nº 01/2020 do Instituto de Matemática e Estatística (IME/UFBA)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), durante a vigência dos termos de estágio, a instituição cedente poderá ser avaliada em relação às seguintes características:
+* Suas **instalações**;
+* A **adequação** dessas instalações à **formação cultural e profissional** do educando.</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L77" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4506,6 +5848,18 @@
       <c r="I78" t="b">
         <v>1</v>
       </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Olá! Como você está perguntando sobre um anexo específico de uma resolução acadêmica, preciso que você me informe o **nome da resolução ou o assunto específico** a que se refere (por exemplo, regulamento de estágio, TCC, atividades complementares, etc.). 
+Assim que você me der essa informação, poderei consultar o documento correto e verificar qual documento consta no Anexo B para te orientar adequadamente!</t>
+        </is>
+      </c>
+      <c r="K78" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="L78" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4545,6 +5899,20 @@
       <c r="I79" t="b">
         <v>1</v>
       </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>De acordo com a **Resolução Nº 01/2020** do Instituto de Matemática e Estatística da UFBA (IME/UFBA), a lei federal que fundamenta o regulamento de estágio não obrigatório é a **Lei Federal nº 11.788, de 25 de setembro de 2008**. 
+Essa informação consta expressamente no preâmbulo e no Art. 1º do documento:
+* [Resolução Nº 01/2020 do IME/UFBA, pág. 1](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf): O preâmbulo indica que a Congregação do IME/UFBA delibera *"no uso de suas atribuições legais, com base na Lei Federal 11.788 de 25 de setembro de 2008"*.
+* [Resolução Nº 01/2020 do IME/UFBA, pág. 2](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf): O Art. 1º reforça que o estágio é *"como previsto na Lei nº 11.788, de 25 de setembro de 2008"*.</t>
+        </is>
+      </c>
+      <c r="K79" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L79" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4583,6 +5951,17 @@
         <v>1</v>
       </c>
       <c r="I80" t="b">
+        <v>1</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>De acordo com o **Parágrafo Único do Art. 1º do Capítulo I** da [Resolução Nº 01/2020 do Instituto de Matemática e Estatística (IME/UFBA)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), o estágio regulamentado por esta norma possui **caráter não-obrigatório**, ficando a critério do estudante realizá-lo ou não, desde que atenda a todos os requisitos estabelecidos na resolução e nas demais normas em vigor (pág. 2).</t>
+        </is>
+      </c>
+      <c r="K80" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L80" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4628,6 +6007,18 @@
       <c r="I81" t="b">
         <v>1</v>
       </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 3º** do regulamento de estágio, os documentos para concessão de estágio (já assinados pelas demais partes) devem ser apresentados inicialmente ao **Centro de Atendimento à Graduação (CEAG)**. 
+O CEAG fará a verificação da validade do convênio com a instituição cedente e, em seguida, encaminhará a documentação ao Colegiado para conferência e assinatura, conforme detalhado na página 2 da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 1-2](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf).</t>
+        </is>
+      </c>
+      <c r="K81" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L81" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4667,6 +6058,19 @@
         <v>1</v>
       </c>
       <c r="I82" t="b">
+        <v>1</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>De acordo com o **Parágrafo Único do Art. 4º do Capítulo III da Resolução nº 01/2020 do IME/UFBA**, o Termo de Compromisso e o Plano de Estágio devem ser apresentados ao Colegiado com **pelo menos 5 (cinco) dias úteis de antecedência** do início das atividades de estágio, para fins de análise e assinatura, não podendo ser emitidos com datas retroativas.
+Você pode consultar o documento oficial completo através do seguinte link:
+[Resoluções 01 e 02/2020 de Estágio Não Obrigatório do IME, pág. 3](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf).</t>
+        </is>
+      </c>
+      <c r="K82" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L82" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4712,6 +6116,19 @@
       <c r="I83" t="b">
         <v>1</v>
       </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>De acordo com o **Parágrafo Único do Art. 4º do Capítulo III** das normas de estágio, **o Termo de Compromisso e o Plano de Estágio NÃO podem ser emitidos com datas retroativas**. 
+Além disso, a documentação deve ser apresentada ao Colegiado com pelo menos **5 (cinco) dias úteis de antecedência** do início das atividades de estágio para análise e assinatura.
+Para mais detalhes, consulte o documento oficial: [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 3-4](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf).</t>
+        </is>
+      </c>
+      <c r="K83" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L83" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4752,6 +6169,17 @@
       <c r="I84" t="b">
         <v>1</v>
       </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>De acordo com o inciso V do Art. 6º da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 3-4](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf) e com o [Checklist - Estágio Não Obrigatório (pág. 10)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), é exigida especificamente dos estudantes do curso de Bacharelado em Estatística a aprovação na disciplina **MATD38 – Estatística Básica B** (ou componente equivalente) como requisito para a realização de estágio.</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L84" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4792,6 +6220,17 @@
       </c>
       <c r="I85" t="b">
         <v>1</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Desculpe, não posso te ajudar com isso, pois o seu curso de cadastro é **Estatística (Bacharel)** e a sua pergunta refere-se aos estudantes do curso de Ciência da Computação, que está fora do escopo do seu curso de atendimento.</t>
+        </is>
+      </c>
+      <c r="K85" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L85" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="86">
@@ -4837,6 +6276,19 @@
       <c r="I86" t="b">
         <v>1</v>
       </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>De acordo com o **Inciso VII do Art. 6º da [Resolução nº 01/2020 do IME/UFBA (pág. 1 e pág. 1 do checklist)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)**, para a realização de estágio por estudantes dos cursos de Matemática, exige-se a aprovação nas seguintes disciplinas:
+* **MATB33 – Limites e Derivadas** (ou equivalentes)
+* **MATB34 – Geometria Analítica e Álgebra Vetorial** (ou equivalentes)</t>
+        </is>
+      </c>
+      <c r="K86" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L86" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4882,6 +6334,20 @@
       <c r="I87" t="b">
         <v>1</v>
       </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 9º** do Capítulo V da **[Resolução Nº 01/2020 - IME (págs. 2 e 7)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)**, os limites máximos de carga horária para a realização do estágio são:
+* **Carga horária diária:** Máximo de **6 (seis)** horas diárias.
+* **Carga horária semanal:** Máximo de **30 (trinta)** horas semanais.
+O regulamento também estabelece que os horários do estágio devem ser compatíveis com as atividades acadêmicas e que **não é permitido deixar de participar das atividades acadêmicas** para a realização de estágios.</t>
+        </is>
+      </c>
+      <c r="K87" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L87" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -4921,6 +6387,18 @@
         <v>1</v>
       </c>
       <c r="I88" t="b">
+        <v>1</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 10 da [Resolução nº 01/2020 do Instituto de Matemática e Estatística (IME)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)**, que estabelece os critérios complementares para concessão de estágio não obrigatório (conforme a página 2 do documento):
+&gt; *"Art. 10º A vigência da primeira concessão de autorização de estágio será de no máximo seis meses, não admitindo renovação automática, podendo ser prorrogada por intervalos de no máximo seis meses cada, com a apresentação de Termo Aditivo e novo Plano de Estágio, até o máximo de 2 anos em uma mesma instituição cedente."*</t>
+        </is>
+      </c>
+      <c r="K88" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L88" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4970,6 +6448,19 @@
       <c r="I89" t="b">
         <v>1</v>
       </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 10 do Capítulo V** da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 2-3](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), o tempo máximo de duração do estágio em uma mesma instituição cedente é de **2 (dois) anos**. 
+A norma detalha que a vigência da primeira concessão de autorização de estágio é de no máximo seis meses, podendo ser prorrogada por intervalos de até seis meses cada (mediante a apresentação de Termo Aditivo e novo Plano de Estágio) até atingir o limite total de 2 anos na mesma empresa/instituição cedente. 
+O **Parágrafo único** do mesmo artigo ressalva que esse prazo poderá exceder os dois anos apenas quando se tratar de estagiário portador de deficiência.</t>
+        </is>
+      </c>
+      <c r="K89" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L89" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5011,6 +6502,18 @@
       <c r="I90" t="b">
         <v>0</v>
       </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 11º** da [Resolução Nº 01/2020 do Instituto de Matemática e Estatística (IME/UFBA)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf) (pág. 2 do documento), o(a) estagiário(a) tem direito a férias remuneradas de trinta dias após completar **doze meses** de estágio na mesma instituição cedente. 
+Caso o estágio possua duração inferior a um ano, o(a) estudante tem direito ao período de férias proporcional ao tempo de estágio. O texto normativo orienta ainda que as férias devem ocorrer, preferencialmente, no período das férias escolares.</t>
+        </is>
+      </c>
+      <c r="K90" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L90" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5051,6 +6554,18 @@
       </c>
       <c r="I91" t="b">
         <v>0</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 13º do Capítulo VI** da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 2-6](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), o estudante deve apresentar o relatório parcial de estágio **a cada seis meses**. 
+Além disso, o **Inciso I do Art. 16º** do mesmo documento reforça que compete ao estudante apresentar os relatórios de estágio conforme o cronograma estabelecido no Plano de Estágio ou a cada seis meses.</t>
+        </is>
+      </c>
+      <c r="K91" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L91" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="92">
@@ -5094,6 +6609,18 @@
       <c r="I92" t="b">
         <v>0</v>
       </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 13º do Capítulo VI** da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 1-2](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), o prazo limite para o envio do relatório final de estágio ao colegiado é de **30 dias após a conclusão de cada etapa**, independentemente da duração do estágio. 
+Além disso, o **Art. 16º** reforça que compete ao estudante apresentar os relatórios de estágio conforme o cronograma estabelecido no Plano de Estágio ou a cada seis meses.</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L92" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5134,6 +6661,20 @@
         <v>0</v>
       </c>
       <c r="I93" t="b">
+        <v>1</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>De acordo com a regulamentação de estágio do Instituto de Matemática e Estatística da UFBA, a instituição cedente deve indicar um funcionário de seu próprio quadro de pessoal para atuar como Supervisor de Estágio, sendo exigido que essa pessoa possua **formação ou experiência profissional na área do curso** (neste caso, na área de Estatística).
+Conforme estabelecido no documento:
+&gt; *"III. Indicar funcionário de seu quadro de pessoal, com formação ou experiência profissional na área do curso, para atuar como Supervisor de Estágio;"* 
+&gt; — ([Resoluções nº 01 e 02/2020 de Estágio Não Obrigatório do IME, Art. 14º, Inciso III, pág. 5](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)).</t>
+        </is>
+      </c>
+      <c r="K93" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L93" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5189,6 +6730,25 @@
       <c r="I94" t="b">
         <v>0</v>
       </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 15º da Resolução nº 01/2020** do Instituto de Matemática e Estatística (IME/UFBA), que estabelece os critérios para a realização de estágio não-obrigatório, os requisitos para o **Professor Orientador de Estágio** são os seguintes:
+* O docente deve ser **professor do Departamento ao qual o Colegiado do curso esteja vinculado** (ou seja, do Departamento de Estatística).
+* O professor deve estar em **regime de dedicação exclusiva**.
+Além disso, o **Art. 15º** estabelece que compete ao Professor Orientador de Estágio:
+* Tomar conhecimento da resolução de estágio e informá-la à instituição cedente (Art. 15º, inciso I, pág. 5).
+* Acompanhar o cumprimento do Plano de Estágio (Art. 15º, inciso II, pág. 5).
+* Avaliar os Relatórios de Estágio apresentados pelo estudante (Art. 15º, inciso III, pág. 5).
+Você pode consultar o teor completo deste regulamento diretamente no documento oficial:
+[Resoluções nº 01 e 02/2020 - Estágio Não Obrigatório IME, pág. 5](http://colest.ime.ubf.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf) *(Nota: verifique também a portaria e diretrizes complementares no site do [Colegiado de Estatística da UFBA](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf))*</t>
+        </is>
+      </c>
+      <c r="K94" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="L94" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5228,6 +6788,18 @@
         <v>1</v>
       </c>
       <c r="I95" t="b">
+        <v>1</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 17º do Capítulo VIII** da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 5-6](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf):
+O desligamento do estudante da instituição cedente ocorrerá **automaticamente** depois de encerrado o prazo fixado no termo de compromisso.</t>
+        </is>
+      </c>
+      <c r="K95" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="L95" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5277,6 +6849,21 @@
       <c r="I96" t="b">
         <v>1</v>
       </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>De acordo com o **Parágrafo único do Art. 18º do Capítulo VIII** da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME (págs. 1-2)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), no caso de rescisão antecipada do termo de compromisso de estágio, o estudante deverá apresentar os seguintes documentos ao Colegiado:
+1. **Um relatório final** de estágio;
+2. **Uma declaração de término do estágio** disponibilizada pela instituição cedente;
+3. **O termo de rescisão**, conforme o modelo constante no **Anexo C** do regulamento.
+O documento ressalta ainda que a não apresentação desses documentos inviabiliza a assinatura de um novo contrato de estágio pelo Colegiado.</t>
+        </is>
+      </c>
+      <c r="K96" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L96" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5321,6 +6908,21 @@
       <c r="I97" t="b">
         <v>1</v>
       </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 1º da Resolução Nº 02/2020**, este documento estabelece a **suspensão** (até 31 de dezembro de 2022) do **Art. 19** e dos **incisos I e II do Art. 6º** da **Resolução Nº 01/2020** (que dispõe sobre os critérios complementares para a concessão de autorização de estágio não obrigatório aos estudantes dos colegiados de graduação do IME/UFBA). 
+A Resolução Nº 02/2020 determina expressamente que continuam mantidos inalterados o *caput* do Art. 6º e seus demais parágrafos.
+Para mais detalhes sobre as disposições originais e as alterações, você pode consultar os documentos oficiais de origem:
+- [Resolução Nº 02/2020 (IME/UFBA), pág. 1](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)
+- [Resolução Nº 01/2020 (IME/UFBA), págs. 1-2](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)</t>
+        </is>
+      </c>
+      <c r="K97" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="L97" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5363,6 +6965,19 @@
       <c r="I98" t="b">
         <v>1</v>
       </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>De acordo com a [Resolução Nº 01/2020](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), a aprovação ocorreu em duas instâncias e datas distintas:
+1. A deliberação em plenária ocorreu na **252ª sessão ordinária**, realizada em **10 de dezembro de 2019** (conforme preâmbulo da pág. 1).
+2. A aprovação formal e assinatura no Gabinete do Diretor do Instituto de Matemática e Estatística (IME/UFBA) ocorreu em **22 de setembro de 2020** (conforme o Art. 2º e a assinatura na pág. 1, além da emissão registrada no SIPAC na pág. 2 do documento [Resolucoes_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, págs. 1-2](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf)).</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="L98" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5406,6 +7021,19 @@
       <c r="I99" t="b">
         <v>0</v>
       </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>**Não, não é permitido** realizar estágio em uma área diferente da área do curso do estudante. 
+De acordo com o **Art. 8º do Capítulo V** da [Resoluções_01_e_02_2020_Estagio_Nao_Obrigatorio_IME, pág. 2](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf):
+&gt; *"O estágio deve estar diretamente relacionado com a área do curso, não sendo permitido realizar estágio em outra área."*</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="L99" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5445,6 +7073,19 @@
         <v>1</v>
       </c>
       <c r="I100" t="b">
+        <v>1</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 12º** do regulamento do Instituto de Matemática e Estatística (IME/UFBA), caso seja necessário alterar informações no decorrer do estágio (tais como horários do exercício de estágio, atividades exercidas, valores da bolsa, prorrogação, entre outros), é obrigatório emitir um **Termo Aditivo e um novo Plano de Estágio**. 
+Além disso, conforme o **Parágrafo único** do mesmo artigo, você deve solicitar à instituição cedente a emissão desses documentos e apresentá-los ao Colegiado **antes** da implementação das alterações previstas.
+Para mais detalhes, consulte o texto completo na [Resolução nº 01/2020 de Estágio Não Obrigatório do IME (págs. 2-3)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf).</t>
+        </is>
+      </c>
+      <c r="K100" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="L100" t="b">
         <v>1</v>
       </c>
     </row>
@@ -5502,6 +7143,18 @@
       <c r="I101" t="b">
         <v>0</v>
       </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>De acordo com o **Art. 7º** da [Resolução nº 01/2020 do IME/UFBA (pág. 1)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf), no caso de renovação de estágio, além do novo Plano de Estágio, é exigida a apresentação de um **Termo Aditivo**.
+Além disso, o **Checklist - Estágio Não Obrigatório** presente no mesmo documento aponta que, por ocasião do termo aditivo, o discente também deve apresentar o **relatório do período estagiado** anterior conforme verificado no [Checklist de Estágio Não Obrigatório da Resolução nº 01/2020 do IME/UFBA (pág. 10)](http://colest.ime.ufba.br/wp-content/uploads/2021/01/Resolucoes_01_e_02_2020_Estagio_nao_obrigatorio_IME.pdf).</t>
+        </is>
+      </c>
+      <c r="K101" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="L101" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>